<commit_message>
Commit 05.1. Creeper Completo
</commit_message>
<xml_diff>
--- a/capas.xlsx
+++ b/capas.xlsx
@@ -19,7 +19,7 @@
     <sheet name="SHORT" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="BRAZOS" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="CAMISA" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="Hoja12" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="CREEPER" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="38">
   <si>
     <t xml:space="preserve">CAPA</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t xml:space="preserve">DETALLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CREEPER</t>
   </si>
   <si>
     <t xml:space="preserve">(50, 100, 100, 50)</t>
@@ -6060,10 +6063,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D152"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="16.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="21.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.86"/>
   </cols>
   <sheetData>
@@ -6072,10 +6075,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6317,6 +6320,976 @@
       </c>
       <c r="B31" s="16" t="n">
         <v>-465.64</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" s="1" t="str">
+        <f aca="false">D1</f>
+        <v>(50, 100, 100, 50)</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="n">
+        <v>492.86</v>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>-461.6</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="n">
+        <v>490.04</v>
+      </c>
+      <c r="B38" s="16" t="n">
+        <v>-474.12</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="n">
+        <v>486.52</v>
+      </c>
+      <c r="B39" s="16" t="n">
+        <v>-488.01</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="15" t="n">
+        <v>481.72</v>
+      </c>
+      <c r="B40" s="16" t="n">
+        <v>-505.06</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="15" t="n">
+        <v>477.44</v>
+      </c>
+      <c r="B41" s="16" t="n">
+        <v>-518.86</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="15" t="n">
+        <v>473.92</v>
+      </c>
+      <c r="B42" s="16" t="n">
+        <v>-526.49</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="15" t="n">
+        <v>461.06</v>
+      </c>
+      <c r="B43" s="16" t="n">
+        <v>-528.55</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="15" t="n">
+        <v>449.15</v>
+      </c>
+      <c r="B44" s="16" t="n">
+        <v>-529.66</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15" t="n">
+        <v>440</v>
+      </c>
+      <c r="B45" s="16" t="n">
+        <v>-530</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="15" t="n">
+        <v>431.32</v>
+      </c>
+      <c r="B46" s="16" t="n">
+        <v>-527.95</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="15" t="n">
+        <v>425.83</v>
+      </c>
+      <c r="B47" s="16" t="n">
+        <v>-526.84</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="15" t="n">
+        <v>427.89</v>
+      </c>
+      <c r="B48" s="16" t="n">
+        <v>-524.26</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="15" t="n">
+        <v>430</v>
+      </c>
+      <c r="B49" s="16" t="n">
+        <v>-520</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="15" t="n">
+        <v>431.92</v>
+      </c>
+      <c r="B50" s="16" t="n">
+        <v>-513.55</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="15" t="n">
+        <v>435.35</v>
+      </c>
+      <c r="B51" s="16" t="n">
+        <v>-502.41</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="15" t="n">
+        <v>437.32</v>
+      </c>
+      <c r="B52" s="16" t="n">
+        <v>-493.66</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="15" t="n">
+        <v>439.55</v>
+      </c>
+      <c r="B53" s="16" t="n">
+        <v>-482.35</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="15" t="n">
+        <v>441.61</v>
+      </c>
+      <c r="B54" s="16" t="n">
+        <v>-473.26</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="15" t="n">
+        <v>441.43</v>
+      </c>
+      <c r="B55" s="16" t="n">
+        <v>-469.49</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="15" t="n">
+        <v>448.03</v>
+      </c>
+      <c r="B56" s="16" t="n">
+        <v>-467.86</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="15" t="n">
+        <v>452.66</v>
+      </c>
+      <c r="B57" s="16" t="n">
+        <v>-469.23</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="15" t="n">
+        <v>459.01</v>
+      </c>
+      <c r="B58" s="16" t="n">
+        <v>-469.49</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="15" t="n">
+        <v>465.69</v>
+      </c>
+      <c r="B59" s="16" t="n">
+        <v>-468.2</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="15" t="n">
+        <v>475</v>
+      </c>
+      <c r="B60" s="16" t="n">
+        <v>-465</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="15" t="n">
+        <v>484.12</v>
+      </c>
+      <c r="B61" s="16" t="n">
+        <v>-462.98</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B64" s="1" t="str">
+        <f aca="false">D1</f>
+        <v>(50, 100, 100, 50)</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="15" t="n">
+        <v>426.74</v>
+      </c>
+      <c r="B67" s="16" t="n">
+        <v>-526.43</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="15" t="n">
+        <v>421.49</v>
+      </c>
+      <c r="B68" s="16" t="n">
+        <v>-541.9</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="15" t="n">
+        <v>417.51</v>
+      </c>
+      <c r="B69" s="16" t="n">
+        <v>-555.79</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="15" t="n">
+        <v>417.73</v>
+      </c>
+      <c r="B70" s="16" t="n">
+        <v>-557.59</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="15" t="n">
+        <v>419.98</v>
+      </c>
+      <c r="B71" s="16" t="n">
+        <v>-558.79</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="15" t="n">
+        <v>435.45</v>
+      </c>
+      <c r="B72" s="16" t="n">
+        <v>-559.27</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="15" t="n">
+        <v>441.86</v>
+      </c>
+      <c r="B73" s="16" t="n">
+        <v>-560.38</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="15" t="n">
+        <v>440.86</v>
+      </c>
+      <c r="B74" s="16" t="n">
+        <v>-585.39</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="15" t="n">
+        <v>439.58</v>
+      </c>
+      <c r="B75" s="16" t="n">
+        <v>-594.03</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="15" t="n">
+        <v>435</v>
+      </c>
+      <c r="B76" s="16" t="n">
+        <v>-605</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="15" t="n">
+        <v>432.41</v>
+      </c>
+      <c r="B77" s="16" t="n">
+        <v>-610.26</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="15" t="n">
+        <v>431.39</v>
+      </c>
+      <c r="B78" s="16" t="n">
+        <v>-616.32</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="15" t="n">
+        <v>429</v>
+      </c>
+      <c r="B79" s="16" t="n">
+        <v>-621.68</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="15" t="n">
+        <v>424.22</v>
+      </c>
+      <c r="B80" s="16" t="n">
+        <v>-629.68</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="15" t="n">
+        <v>420.29</v>
+      </c>
+      <c r="B81" s="16" t="n">
+        <v>-636.82</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="15" t="n">
+        <v>415.95</v>
+      </c>
+      <c r="B82" s="16" t="n">
+        <v>-639.28</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="15" t="n">
+        <v>409.71</v>
+      </c>
+      <c r="B83" s="16" t="n">
+        <v>-641.42</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="15" t="n">
+        <v>400.81</v>
+      </c>
+      <c r="B84" s="16" t="n">
+        <v>-642.49</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="15" t="n">
+        <v>393.39</v>
+      </c>
+      <c r="B85" s="16" t="n">
+        <v>-642.19</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="15" t="n">
+        <v>384.01</v>
+      </c>
+      <c r="B86" s="16" t="n">
+        <v>-639.76</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="15" t="n">
+        <v>385.91</v>
+      </c>
+      <c r="B87" s="16" t="n">
+        <v>-638.33</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="15" t="n">
+        <v>390</v>
+      </c>
+      <c r="B88" s="16" t="n">
+        <v>-635</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="15" t="n">
+        <v>393.39</v>
+      </c>
+      <c r="B89" s="16" t="n">
+        <v>-630.44</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="15" t="n">
+        <v>396.18</v>
+      </c>
+      <c r="B90" s="16" t="n">
+        <v>-624.56</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="15" t="n">
+        <v>402.77</v>
+      </c>
+      <c r="B91" s="16" t="n">
+        <v>-606.15</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="15" t="n">
+        <v>406.51</v>
+      </c>
+      <c r="B92" s="16" t="n">
+        <v>-594.87</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="15" t="n">
+        <v>410.72</v>
+      </c>
+      <c r="B93" s="16" t="n">
+        <v>-583.95</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="15" t="n">
+        <v>410.28</v>
+      </c>
+      <c r="B94" s="16" t="n">
+        <v>-582.44</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="15" t="n">
+        <v>405.74</v>
+      </c>
+      <c r="B95" s="16" t="n">
+        <v>-582.93</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="15" t="n">
+        <v>394.95</v>
+      </c>
+      <c r="B96" s="16" t="n">
+        <v>-583</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="15" t="n">
+        <v>389.16</v>
+      </c>
+      <c r="B97" s="16" t="n">
+        <v>-582.79</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="15" t="n">
+        <v>380.16</v>
+      </c>
+      <c r="B98" s="16" t="n">
+        <v>-581.57</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="15" t="n">
+        <v>372.94</v>
+      </c>
+      <c r="B99" s="16" t="n">
+        <v>-583.04</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="15" t="n">
+        <v>365</v>
+      </c>
+      <c r="B100" s="16" t="n">
+        <v>-585</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="15" t="n">
+        <v>358.88</v>
+      </c>
+      <c r="B101" s="16" t="n">
+        <v>-586.86</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="15" t="n">
+        <v>353.05</v>
+      </c>
+      <c r="B102" s="16" t="n">
+        <v>-588.57</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="15" t="n">
+        <v>345.46</v>
+      </c>
+      <c r="B103" s="16" t="n">
+        <v>-589.1</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="15" t="n">
+        <v>339.7</v>
+      </c>
+      <c r="B104" s="16" t="n">
+        <v>-588.81</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="15" t="n">
+        <v>337.86</v>
+      </c>
+      <c r="B105" s="16" t="n">
+        <v>-593.28</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="15" t="n">
+        <v>334.13</v>
+      </c>
+      <c r="B106" s="16" t="n">
+        <v>-600.93</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="15" t="n">
+        <v>330.01</v>
+      </c>
+      <c r="B107" s="16" t="n">
+        <v>-607.91</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="15" t="n">
+        <v>325.56</v>
+      </c>
+      <c r="B108" s="16" t="n">
+        <v>-613.63</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="15" t="n">
+        <v>322.3</v>
+      </c>
+      <c r="B109" s="16" t="n">
+        <v>-618.48</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="15" t="n">
+        <v>315.85</v>
+      </c>
+      <c r="B110" s="16" t="n">
+        <v>-626.39</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="15" t="n">
+        <v>311.53</v>
+      </c>
+      <c r="B111" s="16" t="n">
+        <v>-630.78</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="15" t="n">
+        <v>305.61</v>
+      </c>
+      <c r="B112" s="16" t="n">
+        <v>-634.11</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="15" t="n">
+        <v>299.82</v>
+      </c>
+      <c r="B113" s="16" t="n">
+        <v>-632.38</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="15" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="B114" s="16" t="n">
+        <v>-631.91</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="15" t="n">
+        <v>289.78</v>
+      </c>
+      <c r="B115" s="16" t="n">
+        <v>-632.38</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="15" t="n">
+        <v>284.06</v>
+      </c>
+      <c r="B116" s="16" t="n">
+        <v>-633.77</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="15" t="n">
+        <v>280.07</v>
+      </c>
+      <c r="B117" s="16" t="n">
+        <v>-633.04</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="15" t="n">
+        <v>279.21</v>
+      </c>
+      <c r="B118" s="16" t="n">
+        <v>-631.91</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="15" t="n">
+        <v>281.87</v>
+      </c>
+      <c r="B119" s="16" t="n">
+        <v>-629.25</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="15" t="n">
+        <v>289.52</v>
+      </c>
+      <c r="B120" s="16" t="n">
+        <v>-621.14</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="15" t="n">
+        <v>291.51</v>
+      </c>
+      <c r="B121" s="16" t="n">
+        <v>-610.35</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="15" t="n">
+        <v>295.9</v>
+      </c>
+      <c r="B122" s="16" t="n">
+        <v>-611.57</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="B123" s="16" t="n">
+        <v>-605</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="15" t="n">
+        <v>304.74</v>
+      </c>
+      <c r="B124" s="16" t="n">
+        <v>-598.73</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="15" t="n">
+        <v>307.74</v>
+      </c>
+      <c r="B125" s="16" t="n">
+        <v>-593.48</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="15" t="n">
+        <v>311.53</v>
+      </c>
+      <c r="B126" s="16" t="n">
+        <v>-586.17</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="15" t="n">
+        <v>313.85</v>
+      </c>
+      <c r="B127" s="16" t="n">
+        <v>-579.32</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="15" t="n">
+        <v>316.71</v>
+      </c>
+      <c r="B128" s="16" t="n">
+        <v>-571.67</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="15" t="n">
+        <v>317.64</v>
+      </c>
+      <c r="B129" s="16" t="n">
+        <v>-567.75</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="15" t="n">
+        <v>323.43</v>
+      </c>
+      <c r="B130" s="16" t="n">
+        <v>-568.34</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="15" t="n">
+        <v>332.67</v>
+      </c>
+      <c r="B131" s="16" t="n">
+        <v>-568.68</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="15" t="n">
+        <v>338.79</v>
+      </c>
+      <c r="B132" s="16" t="n">
+        <v>-568.15</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="15" t="n">
+        <v>342.25</v>
+      </c>
+      <c r="B133" s="16" t="n">
+        <v>-567.55</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="15" t="n">
+        <v>344.04</v>
+      </c>
+      <c r="B134" s="16" t="n">
+        <v>-566.15</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="15" t="n">
+        <v>346.15</v>
+      </c>
+      <c r="B135" s="16" t="n">
+        <v>-563.26</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="15" t="n">
+        <v>349.42</v>
+      </c>
+      <c r="B136" s="16" t="n">
+        <v>-553.28</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="15" t="n">
+        <v>352.31</v>
+      </c>
+      <c r="B137" s="16" t="n">
+        <v>-545.07</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="15" t="n">
+        <v>353.94</v>
+      </c>
+      <c r="B138" s="16" t="n">
+        <v>-538.41</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="15" t="n">
+        <v>354.63</v>
+      </c>
+      <c r="B139" s="16" t="n">
+        <v>-534.55</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="15" t="n">
+        <v>356.89</v>
+      </c>
+      <c r="B140" s="16" t="n">
+        <v>-531.15</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="15" t="n">
+        <v>359.52</v>
+      </c>
+      <c r="B141" s="16" t="n">
+        <v>-531.34</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="15" t="n">
+        <v>363.78</v>
+      </c>
+      <c r="B142" s="16" t="n">
+        <v>-531.11</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="15" t="n">
+        <v>368.47</v>
+      </c>
+      <c r="B143" s="16" t="n">
+        <v>-530.86</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="15" t="n">
+        <v>374.01</v>
+      </c>
+      <c r="B144" s="16" t="n">
+        <v>-528.66</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="15" t="n">
+        <v>378.79</v>
+      </c>
+      <c r="B145" s="16" t="n">
+        <v>-526.6</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="15" t="n">
+        <v>384.73</v>
+      </c>
+      <c r="B146" s="16" t="n">
+        <v>-525.23</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="15" t="n">
+        <v>391.5</v>
+      </c>
+      <c r="B147" s="16" t="n">
+        <v>-523.21</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="15" t="n">
+        <v>398</v>
+      </c>
+      <c r="B148" s="16" t="n">
+        <v>-522.51</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="15" t="n">
+        <v>403.62</v>
+      </c>
+      <c r="B149" s="16" t="n">
+        <v>-523.17</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="15" t="n">
+        <v>409.34</v>
+      </c>
+      <c r="B150" s="16" t="n">
+        <v>-524.4</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="15" t="n">
+        <v>412.84</v>
+      </c>
+      <c r="B151" s="16" t="n">
+        <v>-525.86</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="15" t="n">
+        <v>417.51</v>
+      </c>
+      <c r="B152" s="16" t="n">
+        <v>-526.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit 05.2 Creeper Ahora si
</commit_message>
<xml_diff>
--- a/capas.xlsx
+++ b/capas.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="SOMBRA_CAMISA" sheetId="1" state="visible" r:id="rId3"/>
@@ -20,6 +20,7 @@
     <sheet name="BRAZOS" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="CAMISA" sheetId="11" state="visible" r:id="rId13"/>
     <sheet name="CREEPER" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="CAMISA_LUZ" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="39">
   <si>
     <t xml:space="preserve">CAPA</t>
   </si>
@@ -145,6 +146,9 @@
   </si>
   <si>
     <t xml:space="preserve">(50, 100, 100, 50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(150, 150, 200, 10)</t>
   </si>
 </sst>
 </file>
@@ -7303,6 +7307,433 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D50"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="17.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.65"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <f aca="false">D1</f>
+        <v>(150, 150, 200, 10)</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="n">
+        <v>144.02</v>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>-341.29</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="n">
+        <v>147.27</v>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>-342.09</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="n">
+        <v>150.68</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>-342.64</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="n">
+        <v>153.54</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>-344.54</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="n">
+        <v>156.15</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>-346.84</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="n">
+        <v>159.25</v>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>-350.57</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="n">
+        <v>160.51</v>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>-351.28</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15" t="n">
+        <v>162.18</v>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>-351.04</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15" t="n">
+        <v>166.62</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>-351.04</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="n">
+        <v>169.24</v>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>-351.28</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15" t="n">
+        <v>173.6</v>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>-351.84</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15" t="n">
+        <v>176.85</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>-353.19</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="15" t="n">
+        <v>179.7</v>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>-353.58</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="15" t="n">
+        <v>183.11</v>
+      </c>
+      <c r="B19" s="16" t="n">
+        <v>-351.84</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15" t="n">
+        <v>202.73</v>
+      </c>
+      <c r="B20" s="16" t="n">
+        <v>-348.07</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15" t="n">
+        <v>224.25</v>
+      </c>
+      <c r="B21" s="16" t="n">
+        <v>-345.09</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15" t="n">
+        <v>235.54</v>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>-343.71</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="n">
+        <v>245.99</v>
+      </c>
+      <c r="B23" s="16" t="n">
+        <v>-336.79</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="n">
+        <v>256.6</v>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>-330.7</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15" t="n">
+        <v>261.25</v>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>-329.6</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15" t="n">
+        <v>265.9</v>
+      </c>
+      <c r="B26" s="16" t="n">
+        <v>-331.38</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15" t="n">
+        <v>270</v>
+      </c>
+      <c r="B27" s="16" t="n">
+        <v>-335</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="n">
+        <v>272.9</v>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>-338.5</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="n">
+        <v>275.88</v>
+      </c>
+      <c r="B29" s="16" t="n">
+        <v>-336.62</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15" t="n">
+        <v>280.31</v>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>-336.95</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="n">
+        <v>287.82</v>
+      </c>
+      <c r="B31" s="16" t="n">
+        <v>-338.94</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="n">
+        <v>298.1</v>
+      </c>
+      <c r="B32" s="16" t="n">
+        <v>-342.81</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="15" t="n">
+        <v>301.31</v>
+      </c>
+      <c r="B33" s="16" t="n">
+        <v>-337.5</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15" t="n">
+        <v>324.52</v>
+      </c>
+      <c r="B34" s="16" t="n">
+        <v>-330.1</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15" t="n">
+        <v>321.53</v>
+      </c>
+      <c r="B35" s="16" t="n">
+        <v>-333.41</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="n">
+        <v>314.35</v>
+      </c>
+      <c r="B36" s="16" t="n">
+        <v>-339.16</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="n">
+        <v>307.83</v>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>-342.26</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="n">
+        <v>303.3</v>
+      </c>
+      <c r="B38" s="16" t="n">
+        <v>-350.55</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="n">
+        <v>301.64</v>
+      </c>
+      <c r="B39" s="16" t="n">
+        <v>-354.52</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="15" t="n">
+        <v>280</v>
+      </c>
+      <c r="B40" s="16" t="n">
+        <v>-350</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="15" t="n">
+        <v>274.56</v>
+      </c>
+      <c r="B41" s="16" t="n">
+        <v>-345.46</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="15" t="n">
+        <v>272.35</v>
+      </c>
+      <c r="B42" s="16" t="n">
+        <v>-349.66</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="15" t="n">
+        <v>257.64</v>
+      </c>
+      <c r="B43" s="16" t="n">
+        <v>-349.62</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="15" t="n">
+        <v>250.99</v>
+      </c>
+      <c r="B44" s="16" t="n">
+        <v>-353.44</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15" t="n">
+        <v>228.54</v>
+      </c>
+      <c r="B45" s="16" t="n">
+        <v>-356.68</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="15" t="n">
+        <v>205.85</v>
+      </c>
+      <c r="B46" s="16" t="n">
+        <v>-361.12</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="15" t="n">
+        <v>197.79</v>
+      </c>
+      <c r="B47" s="16" t="n">
+        <v>-365.84</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="15" t="n">
+        <v>186.81</v>
+      </c>
+      <c r="B48" s="16" t="n">
+        <v>-366.6</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="15" t="n">
+        <v>169.45</v>
+      </c>
+      <c r="B49" s="16" t="n">
+        <v>-363.51</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="15" t="n">
+        <v>149.94</v>
+      </c>
+      <c r="B50" s="16" t="n">
+        <v>-354.08</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
Commit 05.2. Cabello Reze
</commit_message>
<xml_diff>
--- a/capas.xlsx
+++ b/capas.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="42">
   <si>
     <t xml:space="preserve">CAPA</t>
   </si>
@@ -167,7 +167,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -215,12 +215,6 @@
       <name val="Courier New"/>
       <family val="3"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Courier New"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -271,7 +265,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -324,11 +318,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2331,10 +2321,10 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="n">
+      <c r="A13" s="14" t="n">
         <v>427.1</v>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="14" t="n">
         <v>-344.57</v>
       </c>
       <c r="F13" s="3"/>
@@ -2346,10 +2336,10 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="n">
+      <c r="A14" s="14" t="n">
         <v>430</v>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="14" t="n">
         <v>-350</v>
       </c>
       <c r="F14" s="3"/>
@@ -2361,10 +2351,10 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="n">
+      <c r="A15" s="15" t="n">
         <v>482.04</v>
       </c>
-      <c r="B15" s="16" t="n">
+      <c r="B15" s="15" t="n">
         <v>-344.57</v>
       </c>
       <c r="F15" s="3"/>
@@ -2494,10 +2484,10 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="n">
+      <c r="A24" s="14" t="n">
         <v>475.54</v>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B24" s="15" t="n">
         <v>-373.1</v>
       </c>
       <c r="I24" s="3" t="n">
@@ -2508,10 +2498,10 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="n">
+      <c r="A25" s="14" t="n">
         <v>475.54</v>
       </c>
-      <c r="B25" s="16" t="n">
+      <c r="B25" s="15" t="n">
         <v>-344.57</v>
       </c>
       <c r="I25" s="3" t="n">
@@ -2522,10 +2512,10 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="n">
+      <c r="A26" s="14" t="n">
         <v>430</v>
       </c>
-      <c r="B26" s="15" t="n">
+      <c r="B26" s="14" t="n">
         <v>-350</v>
       </c>
       <c r="I26" s="3" t="n">
@@ -2759,10 +2749,10 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="16" t="n">
+      <c r="A42" s="15" t="n">
         <v>475.54</v>
       </c>
-      <c r="B42" s="16" t="n">
+      <c r="B42" s="15" t="n">
         <v>-406.99</v>
       </c>
       <c r="G42" s="6"/>
@@ -2774,10 +2764,10 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16" t="n">
+      <c r="A43" s="15" t="n">
         <v>475.54</v>
       </c>
-      <c r="B43" s="16" t="n">
+      <c r="B43" s="15" t="n">
         <v>-373.1</v>
       </c>
       <c r="G43" s="6"/>
@@ -2789,10 +2779,10 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="16" t="n">
+      <c r="A44" s="15" t="n">
         <v>435.33</v>
       </c>
-      <c r="B44" s="16" t="n">
+      <c r="B44" s="15" t="n">
         <v>-373.1</v>
       </c>
       <c r="G44" s="6"/>
@@ -2969,10 +2959,10 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="15" t="n">
+      <c r="A56" s="14" t="n">
         <v>367.74</v>
       </c>
-      <c r="B56" s="16" t="n">
+      <c r="B56" s="15" t="n">
         <v>-420</v>
       </c>
       <c r="H56" s="6"/>
@@ -2984,10 +2974,10 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="16" t="n">
+      <c r="A57" s="15" t="n">
         <v>475.54</v>
       </c>
-      <c r="B57" s="16" t="n">
+      <c r="B57" s="15" t="n">
         <v>-420</v>
       </c>
       <c r="H57" s="6"/>
@@ -2999,10 +2989,10 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="16" t="n">
+      <c r="A58" s="15" t="n">
         <v>475.54</v>
       </c>
-      <c r="B58" s="16" t="n">
+      <c r="B58" s="15" t="n">
         <v>-406.99</v>
       </c>
       <c r="H58" s="6"/>
@@ -3015,10 +3005,10 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="15" t="n">
+      <c r="A59" s="14" t="n">
         <v>401.44</v>
       </c>
-      <c r="B59" s="15" t="n">
+      <c r="B59" s="14" t="n">
         <v>-406.99</v>
       </c>
       <c r="H59" s="6"/>
@@ -3180,10 +3170,10 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="15" t="n">
+      <c r="A70" s="14" t="n">
         <v>300.9</v>
       </c>
-      <c r="B70" s="16" t="n">
+      <c r="B70" s="15" t="n">
         <v>-386.83</v>
       </c>
       <c r="I70" s="3" t="n">
@@ -3194,10 +3184,10 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="16" t="n">
+      <c r="A71" s="15" t="n">
         <v>300.9</v>
       </c>
-      <c r="B71" s="16" t="n">
+      <c r="B71" s="15" t="n">
         <v>-420</v>
       </c>
       <c r="I71" s="3" t="n">
@@ -3208,10 +3198,10 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="15" t="n">
+      <c r="A72" s="14" t="n">
         <v>367.74</v>
       </c>
-      <c r="B72" s="16" t="n">
+      <c r="B72" s="15" t="n">
         <v>-420</v>
       </c>
       <c r="I72" s="3" t="n">
@@ -3403,10 +3393,10 @@
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="16" t="n">
+      <c r="A85" s="15" t="n">
         <v>300.9</v>
       </c>
-      <c r="B85" s="16" t="n">
+      <c r="B85" s="15" t="n">
         <v>-337.8</v>
       </c>
       <c r="G85" s="6"/>
@@ -3418,10 +3408,10 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="16" t="n">
+      <c r="A86" s="15" t="n">
         <v>300.9</v>
       </c>
-      <c r="B86" s="16" t="n">
+      <c r="B86" s="15" t="n">
         <v>-386.83</v>
       </c>
       <c r="G86" s="6"/>
@@ -3433,10 +3423,10 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="15" t="n">
+      <c r="A87" s="14" t="n">
         <v>338.33</v>
       </c>
-      <c r="B87" s="15" t="n">
+      <c r="B87" s="14" t="n">
         <v>-386.83</v>
       </c>
       <c r="G87" s="6"/>
@@ -10528,7 +10518,7 @@
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="0" t="n">
+      <c r="A179" s="12" t="n">
         <v>365.15</v>
       </c>
       <c r="B179" s="3" t="n">
@@ -10542,10 +10532,6 @@
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="11"/>
       <c r="B181" s="11"/>
-    </row>
-    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A182" s="0"/>
-      <c r="B182" s="0"/>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="11"/>
@@ -11970,7 +11956,7 @@
       <c r="A74" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B74" s="13" t="s">
+      <c r="B74" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -12023,26 +12009,26 @@
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0" t="n">
+      <c r="A81" s="12" t="n">
         <v>309.55</v>
       </c>
-      <c r="B81" s="0" t="n">
+      <c r="B81" s="12" t="n">
         <v>-254.93</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="0" t="n">
+      <c r="A82" s="12" t="n">
         <v>294.53</v>
       </c>
-      <c r="B82" s="0" t="n">
+      <c r="B82" s="12" t="n">
         <v>-271.62</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="0" t="n">
+      <c r="A83" s="12" t="n">
         <v>287.45</v>
       </c>
-      <c r="B83" s="0" t="n">
+      <c r="B83" s="12" t="n">
         <v>-273.98</v>
       </c>
     </row>
@@ -12094,7 +12080,7 @@
       <c r="A89" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B89" s="14" t="s">
+      <c r="B89" s="13" t="s">
         <v>10</v>
       </c>
       <c r="C89" s="6"/>
@@ -12241,18 +12227,18 @@
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="0" t="n">
+      <c r="A107" s="12" t="n">
         <v>307.03</v>
       </c>
-      <c r="B107" s="0" t="n">
+      <c r="B107" s="12" t="n">
         <v>-218.95</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="0" t="n">
+      <c r="A108" s="12" t="n">
         <v>268.56</v>
       </c>
-      <c r="B108" s="0" t="n">
+      <c r="B108" s="12" t="n">
         <v>-247.07</v>
       </c>
     </row>
@@ -12444,10 +12430,10 @@
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="0" t="n">
+      <c r="A130" s="12" t="n">
         <v>338.64</v>
       </c>
-      <c r="B130" s="0" t="n">
+      <c r="B130" s="12" t="n">
         <v>-168.14</v>
       </c>
       <c r="D130" s="3" t="n">
@@ -12458,10 +12444,10 @@
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="0" t="n">
+      <c r="A131" s="12" t="n">
         <v>336.66</v>
       </c>
-      <c r="B131" s="0" t="n">
+      <c r="B131" s="12" t="n">
         <v>-154.31</v>
       </c>
       <c r="C131" s="6"/>
@@ -12487,8 +12473,6 @@
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="0"/>
-      <c r="B133" s="0"/>
       <c r="D133" s="3" t="n">
         <v>465.76</v>
       </c>
@@ -12497,8 +12481,6 @@
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="0"/>
-      <c r="B134" s="0"/>
       <c r="D134" s="3" t="n">
         <v>466.18</v>
       </c>
@@ -12507,8 +12489,6 @@
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="0"/>
-      <c r="B135" s="0"/>
       <c r="D135" s="3" t="n">
         <v>465.62</v>
       </c>
@@ -12517,8 +12497,6 @@
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="0"/>
-      <c r="B136" s="0"/>
       <c r="D136" s="3" t="n">
         <v>464.21</v>
       </c>
@@ -12527,8 +12505,6 @@
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="0"/>
-      <c r="B137" s="0"/>
       <c r="D137" s="3" t="n">
         <v>463.36</v>
       </c>
@@ -12537,8 +12513,6 @@
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="0"/>
-      <c r="B138" s="0"/>
       <c r="D138" s="3" t="n">
         <v>462.09</v>
       </c>
@@ -12668,10 +12642,10 @@
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="0" t="n">
+      <c r="A148" s="12" t="n">
         <v>476.98</v>
       </c>
-      <c r="B148" s="0" t="n">
+      <c r="B148" s="12" t="n">
         <v>-201.08</v>
       </c>
       <c r="E148" s="1" t="s">
@@ -12682,10 +12656,10 @@
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="0" t="n">
+      <c r="A149" s="12" t="n">
         <v>477.4</v>
       </c>
-      <c r="B149" s="0" t="n">
+      <c r="B149" s="12" t="n">
         <v>-211.44</v>
       </c>
       <c r="E149" s="1" t="s">
@@ -12994,76 +12968,60 @@
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A186" s="0" t="n">
+      <c r="A186" s="12" t="n">
         <v>445.14</v>
       </c>
-      <c r="B186" s="0" t="n">
+      <c r="B186" s="12" t="n">
         <v>-276.7</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="0" t="n">
+      <c r="A187" s="12" t="n">
         <v>442.49</v>
       </c>
-      <c r="B187" s="0" t="n">
+      <c r="B187" s="12" t="n">
         <v>-272.05</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A188" s="0" t="n">
+      <c r="A188" s="12" t="n">
         <v>430</v>
       </c>
-      <c r="B188" s="0" t="n">
+      <c r="B188" s="12" t="n">
         <v>-260</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A189" s="0" t="n">
+      <c r="A189" s="12" t="n">
         <v>421.95</v>
       </c>
-      <c r="B189" s="0" t="n">
+      <c r="B189" s="12" t="n">
         <v>-264.91</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A190" s="0" t="n">
+      <c r="A190" s="12" t="n">
         <v>424.73</v>
       </c>
-      <c r="B190" s="0" t="n">
+      <c r="B190" s="12" t="n">
         <v>-217.03</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A191" s="0" t="n">
+      <c r="A191" s="12" t="n">
         <v>424.57</v>
       </c>
-      <c r="B191" s="0" t="n">
+      <c r="B191" s="12" t="n">
         <v>-210.38</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A192" s="0" t="n">
+      <c r="A192" s="12" t="n">
         <v>409.81</v>
       </c>
-      <c r="B192" s="0" t="n">
+      <c r="B192" s="12" t="n">
         <v>-194.69</v>
       </c>
-    </row>
-    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A193" s="0"/>
-      <c r="B193" s="0"/>
-    </row>
-    <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A194" s="0"/>
-      <c r="B194" s="0"/>
-    </row>
-    <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A195" s="0"/>
-      <c r="B195" s="0"/>
-    </row>
-    <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A196" s="0"/>
-      <c r="B196" s="0"/>
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="3" t="n">
@@ -13226,10 +13184,10 @@
       </c>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A211" s="0" t="n">
+      <c r="A211" s="12" t="n">
         <v>445.14</v>
       </c>
-      <c r="B211" s="0" t="n">
+      <c r="B211" s="12" t="n">
         <v>-276.7</v>
       </c>
       <c r="E211" s="3" t="n">
@@ -13240,10 +13198,10 @@
       </c>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A212" s="0" t="n">
+      <c r="A212" s="12" t="n">
         <v>442.49</v>
       </c>
-      <c r="B212" s="0" t="n">
+      <c r="B212" s="12" t="n">
         <v>-272.05</v>
       </c>
       <c r="E212" s="3" t="n">
@@ -13268,8 +13226,6 @@
       </c>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A214" s="0"/>
-      <c r="B214" s="0"/>
       <c r="E214" s="3" t="n">
         <v>294.53</v>
       </c>
@@ -13278,8 +13234,6 @@
       </c>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A215" s="0"/>
-      <c r="B215" s="0"/>
       <c r="E215" s="3" t="n">
         <v>300.43</v>
       </c>
@@ -13288,8 +13242,6 @@
       </c>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A216" s="0"/>
-      <c r="B216" s="0"/>
       <c r="E216" s="3" t="n">
         <v>294.29</v>
       </c>
@@ -14774,10 +14726,10 @@
       </c>
     </row>
     <row r="326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A326" s="0" t="n">
+      <c r="A326" s="12" t="n">
         <v>336.66</v>
       </c>
-      <c r="B326" s="0" t="n">
+      <c r="B326" s="12" t="n">
         <v>-154.31</v>
       </c>
       <c r="E326" s="3" t="n">
@@ -14820,7 +14772,7 @@
         <v>2</v>
       </c>
       <c r="B329" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E329" s="3" t="n">
         <v>391.54</v>
@@ -14834,7 +14786,7 @@
         <v>4</v>
       </c>
       <c r="B330" s="1" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E330" s="3" t="n">
         <v>393.32</v>
@@ -14943,10 +14895,10 @@
     </row>
     <row r="338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="3" t="n">
-        <v>400.21</v>
+        <v>387.34</v>
       </c>
       <c r="B338" s="3" t="n">
-        <v>-231.17</v>
+        <v>-228.28</v>
       </c>
       <c r="E338" s="3" t="n">
         <v>411.07</v>
@@ -14957,10 +14909,10 @@
     </row>
     <row r="339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="3" t="n">
-        <v>402.77</v>
+        <v>384.79</v>
       </c>
       <c r="B339" s="3" t="n">
-        <v>-237.04</v>
+        <v>-224.92</v>
       </c>
       <c r="E339" s="3" t="n">
         <v>408.7</v>
@@ -14970,11 +14922,11 @@
       </c>
     </row>
     <row r="340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A340" s="0" t="n">
-        <v>406.6</v>
-      </c>
-      <c r="B340" s="0" t="n">
-        <v>-243.42</v>
+      <c r="A340" s="3" t="n">
+        <v>381.03</v>
+      </c>
+      <c r="B340" s="3" t="n">
+        <v>-221.97</v>
       </c>
       <c r="E340" s="3" t="n">
         <v>406.56</v>
@@ -14984,11 +14936,11 @@
       </c>
     </row>
     <row r="341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A341" s="0" t="n">
-        <v>404.86</v>
-      </c>
-      <c r="B341" s="0" t="n">
-        <v>-247.05</v>
+      <c r="A341" s="3" t="n">
+        <v>377</v>
+      </c>
+      <c r="B341" s="3" t="n">
+        <v>-219.15</v>
       </c>
       <c r="E341" s="3" t="n">
         <v>404.86</v>
@@ -14999,10 +14951,10 @@
     </row>
     <row r="342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="3" t="n">
-        <v>397.43</v>
+        <v>374.58</v>
       </c>
       <c r="B342" s="3" t="n">
-        <v>-247.59</v>
+        <v>-217.27</v>
       </c>
       <c r="E342" s="3" t="n">
         <v>405</v>
@@ -15013,10 +14965,10 @@
     </row>
     <row r="343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="3" t="n">
-        <v>395.99</v>
+        <v>372.16</v>
       </c>
       <c r="B343" s="3" t="n">
-        <v>-243.28</v>
+        <v>-214.98</v>
       </c>
       <c r="E343" s="3" t="n">
         <v>404.86</v>
@@ -15027,10 +14979,10 @@
     </row>
     <row r="344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="3" t="n">
-        <v>394.45</v>
+        <v>368.94</v>
       </c>
       <c r="B344" s="3" t="n">
-        <v>-238.98</v>
+        <v>-211.9</v>
       </c>
       <c r="E344" s="3" t="n">
         <v>405</v>
@@ -15041,10 +14993,10 @@
     </row>
     <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="3" t="n">
-        <v>392.46</v>
+        <v>364.64</v>
       </c>
       <c r="B345" s="3" t="n">
-        <v>-235.89</v>
+        <v>-208.4</v>
       </c>
       <c r="E345" s="3" t="n">
         <v>404.19</v>
@@ -15055,10 +15007,10 @@
     </row>
     <row r="346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A346" s="3" t="n">
-        <v>389.37</v>
+        <v>359.01</v>
       </c>
       <c r="B346" s="3" t="n">
-        <v>-232.69</v>
+        <v>-202.36</v>
       </c>
       <c r="E346" s="3" t="n">
         <v>402.42</v>
@@ -15069,10 +15021,10 @@
     </row>
     <row r="347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A347" s="3" t="n">
-        <v>387.34</v>
+        <v>353.23</v>
       </c>
       <c r="B347" s="3" t="n">
-        <v>-228.28</v>
+        <v>-194.98</v>
       </c>
       <c r="E347" s="3" t="n">
         <v>400.2</v>
@@ -15083,10 +15035,10 @@
     </row>
     <row r="348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A348" s="3" t="n">
-        <v>384.79</v>
+        <v>388.22</v>
       </c>
       <c r="B348" s="3" t="n">
-        <v>-224.92</v>
+        <v>-189.63</v>
       </c>
       <c r="E348" s="3" t="n">
         <v>398.65</v>
@@ -15096,12 +15048,8 @@
       </c>
     </row>
     <row r="349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A349" s="3" t="n">
-        <v>381.03</v>
-      </c>
-      <c r="B349" s="3" t="n">
-        <v>-221.97</v>
-      </c>
+      <c r="A349" s="0"/>
+      <c r="B349" s="0"/>
       <c r="E349" s="3" t="n">
         <v>396.35</v>
       </c>
@@ -15110,12 +15058,8 @@
       </c>
     </row>
     <row r="350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A350" s="3" t="n">
-        <v>377</v>
-      </c>
-      <c r="B350" s="3" t="n">
-        <v>-219.15</v>
-      </c>
+      <c r="A350" s="0"/>
+      <c r="B350" s="0"/>
       <c r="E350" s="3" t="n">
         <v>393.46</v>
       </c>
@@ -15124,12 +15068,8 @@
       </c>
     </row>
     <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A351" s="3" t="n">
-        <v>374.58</v>
-      </c>
-      <c r="B351" s="3" t="n">
-        <v>-217.27</v>
-      </c>
+      <c r="A351" s="0"/>
+      <c r="B351" s="0"/>
       <c r="E351" s="3" t="n">
         <v>390.92</v>
       </c>
@@ -15138,11 +15078,11 @@
       </c>
     </row>
     <row r="352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A352" s="3" t="n">
-        <v>372.16</v>
-      </c>
-      <c r="B352" s="3" t="n">
-        <v>-214.98</v>
+      <c r="A352" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B352" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="E352" s="3" t="n">
         <v>392.68</v>
@@ -15152,11 +15092,11 @@
       </c>
     </row>
     <row r="353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A353" s="3" t="n">
-        <v>368.94</v>
-      </c>
-      <c r="B353" s="3" t="n">
-        <v>-211.9</v>
+      <c r="A353" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B353" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="E353" s="3" t="n">
         <v>395.22</v>
@@ -15166,11 +15106,11 @@
       </c>
     </row>
     <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A354" s="3" t="n">
-        <v>364.64</v>
-      </c>
-      <c r="B354" s="3" t="n">
-        <v>-208.4</v>
+      <c r="A354" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="E354" s="3" t="n">
         <v>397.98</v>
@@ -15180,11 +15120,11 @@
       </c>
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A355" s="3" t="n">
-        <v>359.01</v>
-      </c>
-      <c r="B355" s="3" t="n">
-        <v>-202.36</v>
+      <c r="A355" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B355" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="E355" s="3" t="n">
         <v>398.86</v>
@@ -15194,11 +15134,11 @@
       </c>
     </row>
     <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A356" s="3" t="n">
-        <v>353.23</v>
-      </c>
-      <c r="B356" s="3" t="n">
-        <v>-194.98</v>
+      <c r="A356" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="E356" s="3" t="n">
         <v>398.97</v>
@@ -15209,10 +15149,10 @@
     </row>
     <row r="357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="3" t="n">
-        <v>388.22</v>
+        <v>396.13</v>
       </c>
       <c r="B357" s="3" t="n">
-        <v>-189.63</v>
+        <v>-223.51</v>
       </c>
       <c r="E357" s="3" t="n">
         <v>398.75</v>
@@ -15222,8 +15162,12 @@
       </c>
     </row>
     <row r="358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A358" s="0"/>
-      <c r="B358" s="0"/>
+      <c r="A358" s="3" t="n">
+        <v>400.21</v>
+      </c>
+      <c r="B358" s="3" t="n">
+        <v>-231.17</v>
+      </c>
       <c r="E358" s="3" t="n">
         <v>397.43</v>
       </c>
@@ -15232,8 +15176,12 @@
       </c>
     </row>
     <row r="359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A359" s="0"/>
-      <c r="B359" s="0"/>
+      <c r="A359" s="3" t="n">
+        <v>402.77</v>
+      </c>
+      <c r="B359" s="3" t="n">
+        <v>-237.04</v>
+      </c>
       <c r="E359" s="3" t="n">
         <v>395.99</v>
       </c>
@@ -15242,8 +15190,12 @@
       </c>
     </row>
     <row r="360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A360" s="0"/>
-      <c r="B360" s="0"/>
+      <c r="A360" s="12" t="n">
+        <v>406.6</v>
+      </c>
+      <c r="B360" s="12" t="n">
+        <v>-243.42</v>
+      </c>
       <c r="E360" s="3" t="n">
         <v>394.45</v>
       </c>
@@ -15252,8 +15204,12 @@
       </c>
     </row>
     <row r="361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A361" s="0"/>
-      <c r="B361" s="0"/>
+      <c r="A361" s="12" t="n">
+        <v>404.86</v>
+      </c>
+      <c r="B361" s="12" t="n">
+        <v>-247.05</v>
+      </c>
       <c r="E361" s="3" t="n">
         <v>392.46</v>
       </c>
@@ -15262,8 +15218,12 @@
       </c>
     </row>
     <row r="362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A362" s="0"/>
-      <c r="B362" s="0"/>
+      <c r="A362" s="3" t="n">
+        <v>397.43</v>
+      </c>
+      <c r="B362" s="3" t="n">
+        <v>-247.59</v>
+      </c>
       <c r="E362" s="3" t="n">
         <v>389.37</v>
       </c>
@@ -15272,6 +15232,12 @@
       </c>
     </row>
     <row r="363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A363" s="3" t="n">
+        <v>395.99</v>
+      </c>
+      <c r="B363" s="3" t="n">
+        <v>-243.28</v>
+      </c>
       <c r="E363" s="3" t="n">
         <v>387.34</v>
       </c>
@@ -15280,6 +15246,12 @@
       </c>
     </row>
     <row r="364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A364" s="3" t="n">
+        <v>394.45</v>
+      </c>
+      <c r="B364" s="3" t="n">
+        <v>-238.98</v>
+      </c>
       <c r="E364" s="3" t="n">
         <v>384.79</v>
       </c>
@@ -15288,6 +15260,12 @@
       </c>
     </row>
     <row r="365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A365" s="3" t="n">
+        <v>392.46</v>
+      </c>
+      <c r="B365" s="3" t="n">
+        <v>-235.89</v>
+      </c>
       <c r="E365" s="3" t="n">
         <v>381.03</v>
       </c>
@@ -15296,6 +15274,12 @@
       </c>
     </row>
     <row r="366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A366" s="3" t="n">
+        <v>389.37</v>
+      </c>
+      <c r="B366" s="3" t="n">
+        <v>-232.69</v>
+      </c>
       <c r="E366" s="3" t="n">
         <v>377</v>
       </c>
@@ -15304,6 +15288,12 @@
       </c>
     </row>
     <row r="367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A367" s="0" t="n">
+        <v>387.34</v>
+      </c>
+      <c r="B367" s="0" t="n">
+        <v>-228.28</v>
+      </c>
       <c r="E367" s="3" t="n">
         <v>374.58</v>
       </c>
@@ -15312,6 +15302,12 @@
       </c>
     </row>
     <row r="368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A368" s="0" t="n">
+        <v>384.79</v>
+      </c>
+      <c r="B368" s="0" t="n">
+        <v>-224.92</v>
+      </c>
       <c r="E368" s="3" t="n">
         <v>372.16</v>
       </c>
@@ -15320,6 +15316,12 @@
       </c>
     </row>
     <row r="369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A369" s="3" t="n">
+        <v>396.13</v>
+      </c>
+      <c r="B369" s="3" t="n">
+        <v>-223.51</v>
+      </c>
       <c r="E369" s="3" t="n">
         <v>368.94</v>
       </c>
@@ -15328,6 +15330,10 @@
       </c>
     </row>
     <row r="370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A370" s="0"/>
+      <c r="B370" s="0"/>
+      <c r="C370" s="3"/>
+      <c r="D370" s="3"/>
       <c r="E370" s="3" t="n">
         <v>364.64</v>
       </c>
@@ -15336,6 +15342,10 @@
       </c>
     </row>
     <row r="371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A371" s="0"/>
+      <c r="B371" s="0"/>
+      <c r="C371" s="3"/>
+      <c r="D371" s="3"/>
       <c r="E371" s="3" t="n">
         <v>359.01</v>
       </c>
@@ -15344,6 +15354,10 @@
       </c>
     </row>
     <row r="372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A372" s="0"/>
+      <c r="B372" s="0"/>
+      <c r="C372" s="3"/>
+      <c r="D372" s="3"/>
       <c r="E372" s="3" t="n">
         <v>353.23</v>
       </c>
@@ -15352,6 +15366,10 @@
       </c>
     </row>
     <row r="373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A373" s="0"/>
+      <c r="B373" s="0"/>
+      <c r="C373" s="3"/>
+      <c r="D373" s="3"/>
       <c r="E373" s="3" t="n">
         <v>344.5</v>
       </c>
@@ -15360,6 +15378,10 @@
       </c>
     </row>
     <row r="374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A374" s="0"/>
+      <c r="B374" s="0"/>
+      <c r="C374" s="3"/>
+      <c r="D374" s="3"/>
       <c r="E374" s="3" t="n">
         <v>340.18</v>
       </c>
@@ -15368,6 +15390,10 @@
       </c>
     </row>
     <row r="375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A375" s="0"/>
+      <c r="B375" s="0"/>
+      <c r="C375" s="3"/>
+      <c r="D375" s="3"/>
       <c r="E375" s="3" t="n">
         <v>338.64</v>
       </c>
@@ -15376,6 +15402,10 @@
       </c>
     </row>
     <row r="376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A376" s="0"/>
+      <c r="B376" s="0"/>
+      <c r="C376" s="3"/>
+      <c r="D376" s="3"/>
       <c r="E376" s="3" t="n">
         <v>336.66</v>
       </c>
@@ -15384,6 +15414,10 @@
       </c>
     </row>
     <row r="377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A377" s="0"/>
+      <c r="B377" s="0"/>
+      <c r="C377" s="3"/>
+      <c r="D377" s="3"/>
       <c r="E377" s="3" t="n">
         <v>334.72</v>
       </c>
@@ -15392,6 +15426,10 @@
       </c>
     </row>
     <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A378" s="0"/>
+      <c r="B378" s="0"/>
+      <c r="C378" s="3"/>
+      <c r="D378" s="3"/>
       <c r="E378" s="3" t="n">
         <v>333.18</v>
       </c>

</xml_diff>

<commit_message>
Commit 08.1. Anima Frame 8
</commit_message>
<xml_diff>
--- a/capas.xlsx
+++ b/capas.xlsx
@@ -11293,7 +11293,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G396"/>
+  <dimension ref="A1:G563"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="10.66"/>
@@ -13078,12 +13078,6 @@
       <c r="B203" s="3" t="n">
         <v>-267.72</v>
       </c>
-      <c r="E203" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F203" s="1" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="3" t="n">
@@ -13092,12 +13086,6 @@
       <c r="B204" s="3" t="n">
         <v>-273.26</v>
       </c>
-      <c r="E204" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F204" s="1" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="3" t="n">
@@ -13106,12 +13094,6 @@
       <c r="B205" s="3" t="n">
         <v>-279.88</v>
       </c>
-      <c r="E205" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F205" s="1" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="3" t="n">
@@ -13120,12 +13102,6 @@
       <c r="B206" s="3" t="n">
         <v>-286.7</v>
       </c>
-      <c r="E206" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F206" s="1" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="3" t="n">
@@ -13134,12 +13110,6 @@
       <c r="B207" s="3" t="n">
         <v>-292.87</v>
       </c>
-      <c r="E207" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F207" s="1" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="3" t="n">
@@ -13148,12 +13118,6 @@
       <c r="B208" s="3" t="n">
         <v>-296.86</v>
       </c>
-      <c r="E208" s="3" t="n">
-        <v>335.13</v>
-      </c>
-      <c r="F208" s="3" t="n">
-        <v>-320.95</v>
-      </c>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="3" t="n">
@@ -13162,12 +13126,6 @@
       <c r="B209" s="3" t="n">
         <v>-291.99</v>
       </c>
-      <c r="E209" s="3" t="n">
-        <v>327.81</v>
-      </c>
-      <c r="F209" s="3" t="n">
-        <v>-316.94</v>
-      </c>
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="3" t="n">
@@ -13176,12 +13134,6 @@
       <c r="B210" s="3" t="n">
         <v>-286.23</v>
       </c>
-      <c r="E210" s="3" t="n">
-        <v>320.49</v>
-      </c>
-      <c r="F210" s="3" t="n">
-        <v>-310.1</v>
-      </c>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="n">
@@ -13190,12 +13142,6 @@
       <c r="B211" s="12" t="n">
         <v>-276.7</v>
       </c>
-      <c r="E211" s="3" t="n">
-        <v>315.54</v>
-      </c>
-      <c r="F211" s="3" t="n">
-        <v>-301.83</v>
-      </c>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="12" t="n">
@@ -13204,12 +13150,6 @@
       <c r="B212" s="12" t="n">
         <v>-272.05</v>
       </c>
-      <c r="E212" s="3" t="n">
-        <v>309.4</v>
-      </c>
-      <c r="F212" s="3" t="n">
-        <v>-291.45</v>
-      </c>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="3" t="n">
@@ -13218,36 +13158,6 @@
       <c r="B213" s="3" t="n">
         <v>-267.72</v>
       </c>
-      <c r="E213" s="3" t="n">
-        <v>300</v>
-      </c>
-      <c r="F213" s="3" t="n">
-        <v>-280</v>
-      </c>
-    </row>
-    <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E214" s="3" t="n">
-        <v>294.53</v>
-      </c>
-      <c r="F214" s="3" t="n">
-        <v>-271.62</v>
-      </c>
-    </row>
-    <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E215" s="3" t="n">
-        <v>300.43</v>
-      </c>
-      <c r="F215" s="3" t="n">
-        <v>-286.49</v>
-      </c>
-    </row>
-    <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E216" s="3" t="n">
-        <v>294.29</v>
-      </c>
-      <c r="F216" s="3" t="n">
-        <v>-285.78</v>
-      </c>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="1" t="s">
@@ -13256,12 +13166,6 @@
       <c r="B217" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E217" s="3" t="n">
-        <v>293.58</v>
-      </c>
-      <c r="F217" s="3" t="n">
-        <v>-281.77</v>
-      </c>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="1" t="s">
@@ -13270,12 +13174,6 @@
       <c r="B218" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E218" s="3" t="n">
-        <v>287.45</v>
-      </c>
-      <c r="F218" s="3" t="n">
-        <v>-273.98</v>
-      </c>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="1" t="s">
@@ -13284,12 +13182,6 @@
       <c r="B219" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E219" s="3" t="n">
-        <v>283.2</v>
-      </c>
-      <c r="F219" s="3" t="n">
-        <v>-268.08</v>
-      </c>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="1" t="s">
@@ -13298,12 +13190,6 @@
       <c r="B220" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E220" s="3" t="n">
-        <v>280</v>
-      </c>
-      <c r="F220" s="3" t="n">
-        <v>-260</v>
-      </c>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="1" t="s">
@@ -13312,12 +13198,6 @@
       <c r="B221" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E221" s="3" t="n">
-        <v>274.23</v>
-      </c>
-      <c r="F221" s="3" t="n">
-        <v>-249.2</v>
-      </c>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="3" t="n">
@@ -13326,12 +13206,6 @@
       <c r="B222" s="3" t="n">
         <v>-286.23</v>
       </c>
-      <c r="E222" s="3" t="n">
-        <v>270.69</v>
-      </c>
-      <c r="F222" s="3" t="n">
-        <v>-237.16</v>
-      </c>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="3" t="n">
@@ -13340,12 +13214,6 @@
       <c r="B223" s="3" t="n">
         <v>-276.7</v>
       </c>
-      <c r="E223" s="3" t="n">
-        <v>268.56</v>
-      </c>
-      <c r="F223" s="3" t="n">
-        <v>-232.2</v>
-      </c>
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="3" t="n">
@@ -13354,12 +13222,6 @@
       <c r="B224" s="3" t="n">
         <v>-272.05</v>
       </c>
-      <c r="E224" s="3" t="n">
-        <v>267.62</v>
-      </c>
-      <c r="F224" s="3" t="n">
-        <v>-240.7</v>
-      </c>
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="3" t="n">
@@ -13368,12 +13230,6 @@
       <c r="B225" s="3" t="n">
         <v>-280</v>
       </c>
-      <c r="E225" s="3" t="n">
-        <v>268.56</v>
-      </c>
-      <c r="F225" s="3" t="n">
-        <v>-247.07</v>
-      </c>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="3" t="n">
@@ -13382,12 +13238,6 @@
       <c r="B226" s="3" t="n">
         <v>-287.08</v>
       </c>
-      <c r="E226" s="3" t="n">
-        <v>270.45</v>
-      </c>
-      <c r="F226" s="3" t="n">
-        <v>-254.15</v>
-      </c>
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="3" t="n">
@@ -13396,12 +13246,6 @@
       <c r="B227" s="3" t="n">
         <v>-293.89</v>
       </c>
-      <c r="E227" s="3" t="n">
-        <v>273.99</v>
-      </c>
-      <c r="F227" s="3" t="n">
-        <v>-259.82</v>
-      </c>
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="3" t="n">
@@ -13410,12 +13254,6 @@
       <c r="B228" s="3" t="n">
         <v>-300.7</v>
       </c>
-      <c r="E228" s="3" t="n">
-        <v>276.12</v>
-      </c>
-      <c r="F228" s="3" t="n">
-        <v>-264.3</v>
-      </c>
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="3" t="n">
@@ -13424,12 +13262,6 @@
       <c r="B229" s="3" t="n">
         <v>-306.54</v>
       </c>
-      <c r="E229" s="3" t="n">
-        <v>270.45</v>
-      </c>
-      <c r="F229" s="3" t="n">
-        <v>-261.47</v>
-      </c>
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="3" t="n">
@@ -13438,12 +13270,6 @@
       <c r="B230" s="3" t="n">
         <v>-310.62</v>
       </c>
-      <c r="E230" s="3" t="n">
-        <v>265.97</v>
-      </c>
-      <c r="F230" s="3" t="n">
-        <v>-255.57</v>
-      </c>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="3" t="n">
@@ -13452,12 +13278,6 @@
       <c r="B231" s="3" t="n">
         <v>-314.11</v>
       </c>
-      <c r="E231" s="3" t="n">
-        <v>262.43</v>
-      </c>
-      <c r="F231" s="3" t="n">
-        <v>-249.2</v>
-      </c>
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="3" t="n">
@@ -13466,12 +13286,6 @@
       <c r="B232" s="3" t="n">
         <v>-317.6</v>
       </c>
-      <c r="E232" s="3" t="n">
-        <v>260</v>
-      </c>
-      <c r="F232" s="3" t="n">
-        <v>-240</v>
-      </c>
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="3" t="n">
@@ -13480,12 +13294,6 @@
       <c r="B233" s="3" t="n">
         <v>-323.42</v>
       </c>
-      <c r="E233" s="3" t="n">
-        <v>260.77</v>
-      </c>
-      <c r="F233" s="3" t="n">
-        <v>-227.95</v>
-      </c>
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="3" t="n">
@@ -13494,12 +13302,6 @@
       <c r="B234" s="3" t="n">
         <v>-325.36</v>
       </c>
-      <c r="E234" s="3" t="n">
-        <v>267.48</v>
-      </c>
-      <c r="F234" s="3" t="n">
-        <v>-169.91</v>
-      </c>
     </row>
     <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="3" t="n">
@@ -13510,12 +13312,6 @@
       </c>
       <c r="C235" s="3"/>
       <c r="D235" s="3"/>
-      <c r="E235" s="3" t="n">
-        <v>273.14</v>
-      </c>
-      <c r="F235" s="3" t="n">
-        <v>-151.69</v>
-      </c>
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="3" t="n">
@@ -13526,12 +13322,6 @@
       </c>
       <c r="C236" s="3"/>
       <c r="D236" s="3"/>
-      <c r="E236" s="3" t="n">
-        <v>281.84</v>
-      </c>
-      <c r="F236" s="3" t="n">
-        <v>-136.34</v>
-      </c>
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="3" t="n">
@@ -13542,12 +13332,6 @@
       </c>
       <c r="C237" s="3"/>
       <c r="D237" s="3"/>
-      <c r="E237" s="3" t="n">
-        <v>292.95</v>
-      </c>
-      <c r="F237" s="3" t="n">
-        <v>-120.55</v>
-      </c>
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="3" t="n">
@@ -13558,12 +13342,6 @@
       </c>
       <c r="C238" s="3"/>
       <c r="D238" s="3"/>
-      <c r="E238" s="3" t="n">
-        <v>304.8</v>
-      </c>
-      <c r="F238" s="3" t="n">
-        <v>-108.2</v>
-      </c>
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="3" t="n">
@@ -13574,12 +13352,6 @@
       </c>
       <c r="C239" s="3"/>
       <c r="D239" s="3"/>
-      <c r="E239" s="3" t="n">
-        <v>316.63</v>
-      </c>
-      <c r="F239" s="3" t="n">
-        <v>-99.15</v>
-      </c>
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="3" t="n">
@@ -13590,12 +13362,6 @@
       </c>
       <c r="C240" s="3"/>
       <c r="D240" s="3"/>
-      <c r="E240" s="3" t="n">
-        <v>329.06</v>
-      </c>
-      <c r="F240" s="3" t="n">
-        <v>-92.94</v>
-      </c>
     </row>
     <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="3" t="n">
@@ -13604,12 +13370,6 @@
       <c r="B241" s="3" t="n">
         <v>-279.6</v>
       </c>
-      <c r="E241" s="3" t="n">
-        <v>343.56</v>
-      </c>
-      <c r="F241" s="3" t="n">
-        <v>-92.52</v>
-      </c>
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="3" t="n">
@@ -13618,12 +13378,6 @@
       <c r="B242" s="3" t="n">
         <v>-272.83</v>
       </c>
-      <c r="E242" s="3" t="n">
-        <v>355.99</v>
-      </c>
-      <c r="F242" s="3" t="n">
-        <v>-86.72</v>
-      </c>
     </row>
     <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="3" t="n">
@@ -13632,12 +13386,6 @@
       <c r="B243" s="3" t="n">
         <v>-264.12</v>
       </c>
-      <c r="E243" s="3" t="n">
-        <v>368.01</v>
-      </c>
-      <c r="F243" s="3" t="n">
-        <v>-87.14</v>
-      </c>
     </row>
     <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="3" t="n">
@@ -13646,12 +13394,6 @@
       <c r="B244" s="3" t="n">
         <v>-260</v>
       </c>
-      <c r="E244" s="3" t="n">
-        <v>380.03</v>
-      </c>
-      <c r="F244" s="3" t="n">
-        <v>-88.79</v>
-      </c>
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="1" t="s">
@@ -13660,12 +13402,6 @@
       <c r="B245" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E245" s="3" t="n">
-        <v>391.63</v>
-      </c>
-      <c r="F245" s="3" t="n">
-        <v>-91.28</v>
-      </c>
     </row>
     <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="1" t="s">
@@ -13674,12 +13410,6 @@
       <c r="B246" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E246" s="3" t="n">
-        <v>403.23</v>
-      </c>
-      <c r="F246" s="3" t="n">
-        <v>-95.84</v>
-      </c>
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="1" t="s">
@@ -13688,12 +13418,6 @@
       <c r="B247" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E247" s="3" t="n">
-        <v>412.76</v>
-      </c>
-      <c r="F247" s="3" t="n">
-        <v>-101.22</v>
-      </c>
     </row>
     <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="1" t="s">
@@ -13702,12 +13426,6 @@
       <c r="B248" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E248" s="3" t="n">
-        <v>424.36</v>
-      </c>
-      <c r="F248" s="3" t="n">
-        <v>-107.85</v>
-      </c>
     </row>
     <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="1" t="s">
@@ -13716,12 +13434,6 @@
       <c r="B249" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E249" s="3" t="n">
-        <v>432.23</v>
-      </c>
-      <c r="F249" s="3" t="n">
-        <v>-113.24</v>
-      </c>
     </row>
     <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="3" t="n">
@@ -13730,12 +13442,6 @@
       <c r="B250" s="3" t="n">
         <v>-260</v>
       </c>
-      <c r="E250" s="3" t="n">
-        <v>443.01</v>
-      </c>
-      <c r="F250" s="3" t="n">
-        <v>-122.35</v>
-      </c>
     </row>
     <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="3" t="n">
@@ -13744,12 +13450,6 @@
       <c r="B251" s="3" t="n">
         <v>-267.6</v>
       </c>
-      <c r="E251" s="3" t="n">
-        <v>450.88</v>
-      </c>
-      <c r="F251" s="3" t="n">
-        <v>-131.47</v>
-      </c>
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="3" t="n">
@@ -13758,12 +13458,6 @@
       <c r="B252" s="3" t="n">
         <v>-275.92</v>
       </c>
-      <c r="E252" s="3" t="n">
-        <v>455.44</v>
-      </c>
-      <c r="F252" s="3" t="n">
-        <v>-137.69</v>
-      </c>
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="3" t="n">
@@ -13772,12 +13466,6 @@
       <c r="B253" s="3" t="n">
         <v>-282.31</v>
       </c>
-      <c r="E253" s="3" t="n">
-        <v>461.65</v>
-      </c>
-      <c r="F253" s="3" t="n">
-        <v>-146.39</v>
-      </c>
     </row>
     <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="3" t="n">
@@ -13786,12 +13474,6 @@
       <c r="B254" s="3" t="n">
         <v>-287.53</v>
       </c>
-      <c r="E254" s="3" t="n">
-        <v>468.28</v>
-      </c>
-      <c r="F254" s="3" t="n">
-        <v>-158.4</v>
-      </c>
     </row>
     <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="3" t="n">
@@ -13800,12 +13482,6 @@
       <c r="B255" s="3" t="n">
         <v>-293.92</v>
       </c>
-      <c r="E255" s="3" t="n">
-        <v>470.77</v>
-      </c>
-      <c r="F255" s="3" t="n">
-        <v>-170.42</v>
-      </c>
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="3" t="n">
@@ -13814,12 +13490,6 @@
       <c r="B256" s="3" t="n">
         <v>-275.55</v>
       </c>
-      <c r="E256" s="3" t="n">
-        <v>474.08</v>
-      </c>
-      <c r="F256" s="3" t="n">
-        <v>-180.36</v>
-      </c>
     </row>
     <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="3" t="n">
@@ -13828,12 +13498,6 @@
       <c r="B257" s="3" t="n">
         <v>-264.91</v>
       </c>
-      <c r="E257" s="3" t="n">
-        <v>477.4</v>
-      </c>
-      <c r="F257" s="3" t="n">
-        <v>-191.14</v>
-      </c>
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="3" t="n">
@@ -13842,182 +13506,74 @@
       <c r="B258" s="3" t="n">
         <v>-260</v>
       </c>
-      <c r="E258" s="3" t="n">
-        <v>476.98</v>
-      </c>
-      <c r="F258" s="3" t="n">
-        <v>-201.08</v>
-      </c>
     </row>
     <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="1"/>
       <c r="B259" s="1"/>
-      <c r="E259" s="3" t="n">
-        <v>477.4</v>
-      </c>
-      <c r="F259" s="3" t="n">
-        <v>-211.44</v>
-      </c>
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="1"/>
       <c r="B260" s="1"/>
-      <c r="E260" s="3" t="n">
-        <v>480</v>
-      </c>
-      <c r="F260" s="3" t="n">
-        <v>-220</v>
-      </c>
     </row>
     <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="1"/>
       <c r="B261" s="1"/>
-      <c r="E261" s="3" t="n">
-        <v>478.64</v>
-      </c>
-      <c r="F261" s="3" t="n">
-        <v>-230.5</v>
-      </c>
     </row>
     <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="1"/>
       <c r="B262" s="1"/>
-      <c r="E262" s="3" t="n">
-        <v>477.4</v>
-      </c>
-      <c r="F262" s="3" t="n">
-        <v>-241.69</v>
-      </c>
     </row>
     <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="1"/>
       <c r="B263" s="1"/>
-      <c r="E263" s="3" t="n">
-        <v>476.98</v>
-      </c>
-      <c r="F263" s="3" t="n">
-        <v>-252.46</v>
-      </c>
     </row>
     <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="3"/>
       <c r="B264" s="3"/>
-      <c r="E264" s="3" t="n">
-        <v>473.67</v>
-      </c>
-      <c r="F264" s="3" t="n">
-        <v>-262.4</v>
-      </c>
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="3"/>
       <c r="B265" s="3"/>
-      <c r="E265" s="3" t="n">
-        <v>470.35</v>
-      </c>
-      <c r="F265" s="3" t="n">
-        <v>-271.52</v>
-      </c>
     </row>
     <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="3"/>
       <c r="B266" s="3"/>
-      <c r="E266" s="3" t="n">
-        <v>466.21</v>
-      </c>
-      <c r="F266" s="3" t="n">
-        <v>-281.88</v>
-      </c>
     </row>
     <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="3"/>
       <c r="B267" s="3"/>
-      <c r="E267" s="3" t="n">
-        <v>470.28</v>
-      </c>
-      <c r="F267" s="3" t="n">
-        <v>-266.73</v>
-      </c>
     </row>
     <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="3"/>
       <c r="B268" s="3"/>
-      <c r="E268" s="3" t="n">
-        <v>471.83</v>
-      </c>
-      <c r="F268" s="3" t="n">
-        <v>-258.69</v>
-      </c>
     </row>
     <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="3"/>
       <c r="B269" s="3"/>
-      <c r="E269" s="3" t="n">
-        <v>472.11</v>
-      </c>
-      <c r="F269" s="3" t="n">
-        <v>-249.66</v>
-      </c>
     </row>
     <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="3"/>
       <c r="B270" s="3"/>
-      <c r="E270" s="3" t="n">
-        <v>472.39</v>
-      </c>
-      <c r="F270" s="3" t="n">
-        <v>-240.62</v>
-      </c>
     </row>
     <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="3"/>
       <c r="B271" s="3"/>
-      <c r="E271" s="3" t="n">
-        <v>472.96</v>
-      </c>
-      <c r="F271" s="3" t="n">
-        <v>-232.16</v>
-      </c>
     </row>
     <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="3"/>
       <c r="B272" s="3"/>
-      <c r="E272" s="3" t="n">
-        <v>470.98</v>
-      </c>
-      <c r="F272" s="3" t="n">
-        <v>-223.97</v>
-      </c>
     </row>
     <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="3"/>
       <c r="B273" s="3"/>
-      <c r="E273" s="3" t="n">
-        <v>469.99</v>
-      </c>
-      <c r="F273" s="3" t="n">
-        <v>-216.63</v>
-      </c>
     </row>
     <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="3"/>
       <c r="B274" s="3"/>
-      <c r="E274" s="3" t="n">
-        <v>467.45</v>
-      </c>
-      <c r="F274" s="3" t="n">
-        <v>-209.29</v>
-      </c>
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="3"/>
       <c r="B275" s="3"/>
-      <c r="E275" s="3" t="n">
-        <v>465.76</v>
-      </c>
-      <c r="F275" s="3" t="n">
-        <v>-214.37</v>
-      </c>
     </row>
     <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="1" t="s">
@@ -14026,12 +13582,6 @@
       <c r="B276" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E276" s="3" t="n">
-        <v>466.18</v>
-      </c>
-      <c r="F276" s="3" t="n">
-        <v>-221.71</v>
-      </c>
     </row>
     <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="1" t="s">
@@ -14040,12 +13590,6 @@
       <c r="B277" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E277" s="3" t="n">
-        <v>465.62</v>
-      </c>
-      <c r="F277" s="3" t="n">
-        <v>-228.2</v>
-      </c>
     </row>
     <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="1" t="s">
@@ -14054,12 +13598,6 @@
       <c r="B278" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E278" s="3" t="n">
-        <v>464.21</v>
-      </c>
-      <c r="F278" s="3" t="n">
-        <v>-234.13</v>
-      </c>
     </row>
     <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="1" t="s">
@@ -14068,12 +13606,6 @@
       <c r="B279" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E279" s="3" t="n">
-        <v>463.36</v>
-      </c>
-      <c r="F279" s="3" t="n">
-        <v>-239.21</v>
-      </c>
     </row>
     <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="1" t="s">
@@ -14082,12 +13614,6 @@
       <c r="B280" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E280" s="3" t="n">
-        <v>462.09</v>
-      </c>
-      <c r="F280" s="3" t="n">
-        <v>-244.86</v>
-      </c>
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="3" t="n">
@@ -14096,12 +13622,6 @@
       <c r="B281" s="3" t="n">
         <v>-243.42</v>
       </c>
-      <c r="E281" s="3" t="n">
-        <v>460.4</v>
-      </c>
-      <c r="F281" s="3" t="n">
-        <v>-248.67</v>
-      </c>
     </row>
     <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="3" t="n">
@@ -14110,12 +13630,6 @@
       <c r="B282" s="3" t="n">
         <v>-246.74</v>
       </c>
-      <c r="E282" s="3" t="n">
-        <v>458.42</v>
-      </c>
-      <c r="F282" s="3" t="n">
-        <v>-253.04</v>
-      </c>
     </row>
     <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="3" t="n">
@@ -14124,12 +13638,6 @@
       <c r="B283" s="3" t="n">
         <v>-249.78</v>
       </c>
-      <c r="E283" s="3" t="n">
-        <v>456.59</v>
-      </c>
-      <c r="F283" s="3" t="n">
-        <v>-257.42</v>
-      </c>
     </row>
     <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="3" t="n">
@@ -14138,12 +13646,6 @@
       <c r="B284" s="3" t="n">
         <v>-250</v>
       </c>
-      <c r="E284" s="3" t="n">
-        <v>454.05</v>
-      </c>
-      <c r="F284" s="3" t="n">
-        <v>-262.08</v>
-      </c>
     </row>
     <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="3" t="n">
@@ -14152,12 +13654,6 @@
       <c r="B285" s="3" t="n">
         <v>-250.74</v>
       </c>
-      <c r="E285" s="3" t="n">
-        <v>450.94</v>
-      </c>
-      <c r="F285" s="3" t="n">
-        <v>-267.72</v>
-      </c>
     </row>
     <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="3" t="n">
@@ -14166,12 +13662,6 @@
       <c r="B286" s="3" t="n">
         <v>-249.27</v>
       </c>
-      <c r="E286" s="3" t="n">
-        <v>449.36</v>
-      </c>
-      <c r="F286" s="3" t="n">
-        <v>-273.26</v>
-      </c>
     </row>
     <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="3" t="n">
@@ -14180,12 +13670,6 @@
       <c r="B287" s="3" t="n">
         <v>-247.49</v>
       </c>
-      <c r="E287" s="3" t="n">
-        <v>451.22</v>
-      </c>
-      <c r="F287" s="3" t="n">
-        <v>-279.88</v>
-      </c>
     </row>
     <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="3" t="n">
@@ -14194,12 +13678,6 @@
       <c r="B288" s="3" t="n">
         <v>-247.05</v>
       </c>
-      <c r="E288" s="3" t="n">
-        <v>453.91</v>
-      </c>
-      <c r="F288" s="3" t="n">
-        <v>-286.7</v>
-      </c>
     </row>
     <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="3" t="n">
@@ -14208,12 +13686,6 @@
       <c r="B289" s="3" t="n">
         <v>-250</v>
       </c>
-      <c r="E289" s="3" t="n">
-        <v>455.11</v>
-      </c>
-      <c r="F289" s="3" t="n">
-        <v>-292.87</v>
-      </c>
     </row>
     <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="3" t="n">
@@ -14222,12 +13694,6 @@
       <c r="B290" s="3" t="n">
         <v>-252.74</v>
       </c>
-      <c r="E290" s="3" t="n">
-        <v>457.77</v>
-      </c>
-      <c r="F290" s="3" t="n">
-        <v>-296.86</v>
-      </c>
     </row>
     <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="3" t="n">
@@ -14236,12 +13702,6 @@
       <c r="B291" s="3" t="n">
         <v>-243.42</v>
       </c>
-      <c r="E291" s="3" t="n">
-        <v>451.57</v>
-      </c>
-      <c r="F291" s="3" t="n">
-        <v>-291.99</v>
-      </c>
     </row>
     <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="1" t="s">
@@ -14250,12 +13710,6 @@
       <c r="B292" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E292" s="3" t="n">
-        <v>448.24</v>
-      </c>
-      <c r="F292" s="3" t="n">
-        <v>-286.23</v>
-      </c>
     </row>
     <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="1" t="s">
@@ -14264,12 +13718,6 @@
       <c r="B293" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E293" s="3" t="n">
-        <v>445.14</v>
-      </c>
-      <c r="F293" s="3" t="n">
-        <v>-276.7</v>
-      </c>
     </row>
     <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="1" t="s">
@@ -14278,12 +13726,6 @@
       <c r="B294" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E294" s="3" t="n">
-        <v>442.49</v>
-      </c>
-      <c r="F294" s="3" t="n">
-        <v>-272.05</v>
-      </c>
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="1" t="s">
@@ -14292,12 +13734,6 @@
       <c r="B295" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E295" s="3" t="n">
-        <v>440</v>
-      </c>
-      <c r="F295" s="3" t="n">
-        <v>-280</v>
-      </c>
     </row>
     <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="1" t="s">
@@ -14306,12 +13742,6 @@
       <c r="B296" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E296" s="3" t="n">
-        <v>437.66</v>
-      </c>
-      <c r="F296" s="3" t="n">
-        <v>-287.08</v>
-      </c>
     </row>
     <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="3" t="n">
@@ -14320,12 +13750,6 @@
       <c r="B297" s="3" t="n">
         <v>-252.74</v>
       </c>
-      <c r="E297" s="3" t="n">
-        <v>433.77</v>
-      </c>
-      <c r="F297" s="3" t="n">
-        <v>-293.89</v>
-      </c>
     </row>
     <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="3" t="n">
@@ -14334,12 +13758,6 @@
       <c r="B298" s="3" t="n">
         <v>-255</v>
       </c>
-      <c r="E298" s="3" t="n">
-        <v>429.88</v>
-      </c>
-      <c r="F298" s="3" t="n">
-        <v>-300.7</v>
-      </c>
     </row>
     <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="3" t="n">
@@ -14348,12 +13766,6 @@
       <c r="B299" s="3" t="n">
         <v>-258.58</v>
       </c>
-      <c r="E299" s="3" t="n">
-        <v>425.99</v>
-      </c>
-      <c r="F299" s="3" t="n">
-        <v>-306.54</v>
-      </c>
     </row>
     <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="3" t="n">
@@ -14362,12 +13774,6 @@
       <c r="B300" s="3" t="n">
         <v>-263.17</v>
       </c>
-      <c r="E300" s="3" t="n">
-        <v>422.73</v>
-      </c>
-      <c r="F300" s="3" t="n">
-        <v>-310.62</v>
-      </c>
     </row>
     <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A301" s="3" t="n">
@@ -14376,12 +13782,6 @@
       <c r="B301" s="3" t="n">
         <v>-266.86</v>
       </c>
-      <c r="E301" s="3" t="n">
-        <v>420.02</v>
-      </c>
-      <c r="F301" s="3" t="n">
-        <v>-314.11</v>
-      </c>
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="3" t="n">
@@ -14390,12 +13790,6 @@
       <c r="B302" s="3" t="n">
         <v>-269.9</v>
       </c>
-      <c r="E302" s="3" t="n">
-        <v>417.04</v>
-      </c>
-      <c r="F302" s="3" t="n">
-        <v>-317.6</v>
-      </c>
     </row>
     <row r="303" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="3" t="n">
@@ -14404,12 +13798,6 @@
       <c r="B303" s="3" t="n">
         <v>-273</v>
       </c>
-      <c r="E303" s="3" t="n">
-        <v>409.67</v>
-      </c>
-      <c r="F303" s="3" t="n">
-        <v>-323.42</v>
-      </c>
     </row>
     <row r="304" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="3" t="n">
@@ -14418,12 +13806,6 @@
       <c r="B304" s="3" t="n">
         <v>-276.27</v>
       </c>
-      <c r="E304" s="3" t="n">
-        <v>406.31</v>
-      </c>
-      <c r="F304" s="3" t="n">
-        <v>-325.36</v>
-      </c>
     </row>
     <row r="305" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="3" t="n">
@@ -14432,12 +13814,6 @@
       <c r="B305" s="3" t="n">
         <v>-276.94</v>
       </c>
-      <c r="E305" s="3" t="n">
-        <v>410</v>
-      </c>
-      <c r="F305" s="3" t="n">
-        <v>-320</v>
-      </c>
     </row>
     <row r="306" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="3" t="n">
@@ -14446,12 +13822,6 @@
       <c r="B306" s="3" t="n">
         <v>-273.18</v>
       </c>
-      <c r="E306" s="3" t="n">
-        <v>413.55</v>
-      </c>
-      <c r="F306" s="3" t="n">
-        <v>-313.85</v>
-      </c>
     </row>
     <row r="307" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A307" s="3" t="n">
@@ -14460,12 +13830,6 @@
       <c r="B307" s="3" t="n">
         <v>-269.43</v>
       </c>
-      <c r="E307" s="3" t="n">
-        <v>416.91</v>
-      </c>
-      <c r="F307" s="3" t="n">
-        <v>-308.29</v>
-      </c>
     </row>
     <row r="308" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="3" t="n">
@@ -14474,12 +13838,6 @@
       <c r="B308" s="3" t="n">
         <v>-265.13</v>
       </c>
-      <c r="E308" s="3" t="n">
-        <v>420.53</v>
-      </c>
-      <c r="F308" s="3" t="n">
-        <v>-302.86</v>
-      </c>
     </row>
     <row r="309" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="3" t="n">
@@ -14488,12 +13846,6 @@
       <c r="B309" s="3" t="n">
         <v>-261.27</v>
       </c>
-      <c r="E309" s="3" t="n">
-        <v>423.25</v>
-      </c>
-      <c r="F309" s="3" t="n">
-        <v>-296.78</v>
-      </c>
     </row>
     <row r="310" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="3" t="n">
@@ -14502,12 +13854,6 @@
       <c r="B310" s="3" t="n">
         <v>-256.74</v>
       </c>
-      <c r="E310" s="3" t="n">
-        <v>426.48</v>
-      </c>
-      <c r="F310" s="3" t="n">
-        <v>-286.95</v>
-      </c>
     </row>
     <row r="311" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="3" t="n">
@@ -14516,12 +13862,6 @@
       <c r="B311" s="3" t="n">
         <v>-252.66</v>
       </c>
-      <c r="E311" s="3" t="n">
-        <v>428.22</v>
-      </c>
-      <c r="F311" s="3" t="n">
-        <v>-279.6</v>
-      </c>
     </row>
     <row r="312" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A312" s="3" t="n">
@@ -14530,12 +13870,6 @@
       <c r="B312" s="3" t="n">
         <v>-247.59</v>
       </c>
-      <c r="E312" s="3" t="n">
-        <v>429.77</v>
-      </c>
-      <c r="F312" s="3" t="n">
-        <v>-272.83</v>
-      </c>
     </row>
     <row r="313" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="3" t="n">
@@ -14544,12 +13878,6 @@
       <c r="B313" s="3" t="n">
         <v>-252.74</v>
       </c>
-      <c r="E313" s="3" t="n">
-        <v>430.93</v>
-      </c>
-      <c r="F313" s="3" t="n">
-        <v>-264.12</v>
-      </c>
     </row>
     <row r="314" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="1" t="s">
@@ -14558,12 +13886,6 @@
       <c r="B314" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E314" s="3" t="n">
-        <v>430</v>
-      </c>
-      <c r="F314" s="3" t="n">
-        <v>-260</v>
-      </c>
     </row>
     <row r="315" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A315" s="1" t="s">
@@ -14572,12 +13894,6 @@
       <c r="B315" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E315" s="3" t="n">
-        <v>427.64</v>
-      </c>
-      <c r="F315" s="3" t="n">
-        <v>-267.6</v>
-      </c>
     </row>
     <row r="316" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A316" s="1" t="s">
@@ -14586,12 +13902,6 @@
       <c r="B316" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E316" s="3" t="n">
-        <v>424.16</v>
-      </c>
-      <c r="F316" s="3" t="n">
-        <v>-275.92</v>
-      </c>
     </row>
     <row r="317" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="1" t="s">
@@ -14600,12 +13910,6 @@
       <c r="B317" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E317" s="3" t="n">
-        <v>420.87</v>
-      </c>
-      <c r="F317" s="3" t="n">
-        <v>-282.31</v>
-      </c>
     </row>
     <row r="318" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="1" t="s">
@@ -14614,12 +13918,6 @@
       <c r="B318" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E318" s="3" t="n">
-        <v>418.74</v>
-      </c>
-      <c r="F318" s="3" t="n">
-        <v>-287.53</v>
-      </c>
     </row>
     <row r="319" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A319" s="3" t="n">
@@ -14630,12 +13928,6 @@
       </c>
       <c r="C319" s="3"/>
       <c r="D319" s="3"/>
-      <c r="E319" s="3" t="n">
-        <v>413.71</v>
-      </c>
-      <c r="F319" s="3" t="n">
-        <v>-293.92</v>
-      </c>
     </row>
     <row r="320" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="3" t="n">
@@ -14646,12 +13938,6 @@
       </c>
       <c r="C320" s="3"/>
       <c r="D320" s="3"/>
-      <c r="E320" s="3" t="n">
-        <v>420.04</v>
-      </c>
-      <c r="F320" s="3" t="n">
-        <v>-275.55</v>
-      </c>
     </row>
     <row r="321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="3" t="n">
@@ -14662,12 +13948,6 @@
       </c>
       <c r="C321" s="3"/>
       <c r="D321" s="3"/>
-      <c r="E321" s="3" t="n">
-        <v>421.95</v>
-      </c>
-      <c r="F321" s="3" t="n">
-        <v>-264.91</v>
-      </c>
     </row>
     <row r="322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="3" t="n">
@@ -14676,12 +13956,6 @@
       <c r="B322" s="3" t="n">
         <v>-194.98</v>
       </c>
-      <c r="E322" s="3" t="n">
-        <v>424.73</v>
-      </c>
-      <c r="F322" s="3" t="n">
-        <v>-217.03</v>
-      </c>
     </row>
     <row r="323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="3" t="n">
@@ -14690,12 +13964,6 @@
       <c r="B323" s="3" t="n">
         <v>-181.41</v>
       </c>
-      <c r="E323" s="3" t="n">
-        <v>424.57</v>
-      </c>
-      <c r="F323" s="3" t="n">
-        <v>-210.38</v>
-      </c>
     </row>
     <row r="324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="3" t="n">
@@ -14704,12 +13972,6 @@
       <c r="B324" s="3" t="n">
         <v>-168.14</v>
       </c>
-      <c r="E324" s="3" t="n">
-        <v>409.81</v>
-      </c>
-      <c r="F324" s="3" t="n">
-        <v>-194.69</v>
-      </c>
     </row>
     <row r="325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A325" s="3" t="n">
@@ -14718,12 +13980,6 @@
       <c r="B325" s="3" t="n">
         <v>-163.14</v>
       </c>
-      <c r="E325" s="3" t="n">
-        <v>390.37</v>
-      </c>
-      <c r="F325" s="3" t="n">
-        <v>-167.38</v>
-      </c>
     </row>
     <row r="326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="12" t="n">
@@ -14732,12 +13988,6 @@
       <c r="B326" s="12" t="n">
         <v>-154.31</v>
       </c>
-      <c r="E326" s="3" t="n">
-        <v>389.68</v>
-      </c>
-      <c r="F326" s="3" t="n">
-        <v>-178.19</v>
-      </c>
     </row>
     <row r="327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A327" s="3" t="n">
@@ -14746,12 +13996,6 @@
       <c r="B327" s="3" t="n">
         <v>-167.38</v>
       </c>
-      <c r="E327" s="3" t="n">
-        <v>388.22</v>
-      </c>
-      <c r="F327" s="3" t="n">
-        <v>-189.63</v>
-      </c>
     </row>
     <row r="328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A328" s="1" t="s">
@@ -14760,12 +14004,6 @@
       <c r="B328" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E328" s="3" t="n">
-        <v>390</v>
-      </c>
-      <c r="F328" s="3" t="n">
-        <v>-198.49</v>
-      </c>
     </row>
     <row r="329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A329" s="1" t="s">
@@ -14774,12 +14012,6 @@
       <c r="B329" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E329" s="3" t="n">
-        <v>391.54</v>
-      </c>
-      <c r="F329" s="3" t="n">
-        <v>-206.15</v>
-      </c>
     </row>
     <row r="330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A330" s="1" t="s">
@@ -14788,12 +14020,6 @@
       <c r="B330" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E330" s="3" t="n">
-        <v>393.32</v>
-      </c>
-      <c r="F330" s="3" t="n">
-        <v>-214.57</v>
-      </c>
     </row>
     <row r="331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="1" t="s">
@@ -14802,12 +14028,6 @@
       <c r="B331" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E331" s="3" t="n">
-        <v>396.13</v>
-      </c>
-      <c r="F331" s="3" t="n">
-        <v>-223.51</v>
-      </c>
     </row>
     <row r="332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A332" s="1" t="s">
@@ -14816,12 +14036,6 @@
       <c r="B332" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E332" s="3" t="n">
-        <v>400.21</v>
-      </c>
-      <c r="F332" s="3" t="n">
-        <v>-231.17</v>
-      </c>
     </row>
     <row r="333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A333" s="3" t="n">
@@ -14830,12 +14044,6 @@
       <c r="B333" s="3" t="n">
         <v>-189.63</v>
       </c>
-      <c r="E333" s="3" t="n">
-        <v>402.77</v>
-      </c>
-      <c r="F333" s="3" t="n">
-        <v>-237.04</v>
-      </c>
     </row>
     <row r="334" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="3" t="n">
@@ -14844,12 +14052,6 @@
       <c r="B334" s="3" t="n">
         <v>-198.49</v>
       </c>
-      <c r="E334" s="3" t="n">
-        <v>406.6</v>
-      </c>
-      <c r="F334" s="3" t="n">
-        <v>-243.42</v>
-      </c>
     </row>
     <row r="335" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A335" s="3" t="n">
@@ -14858,12 +14060,6 @@
       <c r="B335" s="3" t="n">
         <v>-206.15</v>
       </c>
-      <c r="E335" s="3" t="n">
-        <v>410.68</v>
-      </c>
-      <c r="F335" s="3" t="n">
-        <v>-246.74</v>
-      </c>
     </row>
     <row r="336" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="3" t="n">
@@ -14872,12 +14068,6 @@
       <c r="B336" s="3" t="n">
         <v>-214.57</v>
       </c>
-      <c r="E336" s="3" t="n">
-        <v>412.33</v>
-      </c>
-      <c r="F336" s="3" t="n">
-        <v>-249.78</v>
-      </c>
     </row>
     <row r="337" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A337" s="3" t="n">
@@ -14886,12 +14076,6 @@
       <c r="B337" s="3" t="n">
         <v>-223.51</v>
       </c>
-      <c r="E337" s="3" t="n">
-        <v>415</v>
-      </c>
-      <c r="F337" s="3" t="n">
-        <v>-250</v>
-      </c>
     </row>
     <row r="338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="3" t="n">
@@ -14900,12 +14084,6 @@
       <c r="B338" s="3" t="n">
         <v>-228.28</v>
       </c>
-      <c r="E338" s="3" t="n">
-        <v>411.07</v>
-      </c>
-      <c r="F338" s="3" t="n">
-        <v>-250.74</v>
-      </c>
     </row>
     <row r="339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="3" t="n">
@@ -14914,12 +14092,6 @@
       <c r="B339" s="3" t="n">
         <v>-224.92</v>
       </c>
-      <c r="E339" s="3" t="n">
-        <v>408.7</v>
-      </c>
-      <c r="F339" s="3" t="n">
-        <v>-249.27</v>
-      </c>
     </row>
     <row r="340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="3" t="n">
@@ -14928,12 +14100,6 @@
       <c r="B340" s="3" t="n">
         <v>-221.97</v>
       </c>
-      <c r="E340" s="3" t="n">
-        <v>406.56</v>
-      </c>
-      <c r="F340" s="3" t="n">
-        <v>-247.49</v>
-      </c>
     </row>
     <row r="341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="3" t="n">
@@ -14942,12 +14108,6 @@
       <c r="B341" s="3" t="n">
         <v>-219.15</v>
       </c>
-      <c r="E341" s="3" t="n">
-        <v>404.86</v>
-      </c>
-      <c r="F341" s="3" t="n">
-        <v>-247.05</v>
-      </c>
     </row>
     <row r="342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="3" t="n">
@@ -14956,12 +14116,6 @@
       <c r="B342" s="3" t="n">
         <v>-217.27</v>
       </c>
-      <c r="E342" s="3" t="n">
-        <v>405</v>
-      </c>
-      <c r="F342" s="3" t="n">
-        <v>-250</v>
-      </c>
     </row>
     <row r="343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="3" t="n">
@@ -14970,12 +14124,6 @@
       <c r="B343" s="3" t="n">
         <v>-214.98</v>
       </c>
-      <c r="E343" s="3" t="n">
-        <v>404.86</v>
-      </c>
-      <c r="F343" s="3" t="n">
-        <v>-252.74</v>
-      </c>
     </row>
     <row r="344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="3" t="n">
@@ -14984,12 +14132,6 @@
       <c r="B344" s="3" t="n">
         <v>-211.9</v>
       </c>
-      <c r="E344" s="3" t="n">
-        <v>405</v>
-      </c>
-      <c r="F344" s="3" t="n">
-        <v>-255</v>
-      </c>
     </row>
     <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="3" t="n">
@@ -14998,12 +14140,6 @@
       <c r="B345" s="3" t="n">
         <v>-208.4</v>
       </c>
-      <c r="E345" s="3" t="n">
-        <v>404.19</v>
-      </c>
-      <c r="F345" s="3" t="n">
-        <v>-258.58</v>
-      </c>
     </row>
     <row r="346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A346" s="3" t="n">
@@ -15012,12 +14148,6 @@
       <c r="B346" s="3" t="n">
         <v>-202.36</v>
       </c>
-      <c r="E346" s="3" t="n">
-        <v>402.42</v>
-      </c>
-      <c r="F346" s="3" t="n">
-        <v>-263.17</v>
-      </c>
     </row>
     <row r="347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A347" s="3" t="n">
@@ -15026,12 +14156,6 @@
       <c r="B347" s="3" t="n">
         <v>-194.98</v>
       </c>
-      <c r="E347" s="3" t="n">
-        <v>400.2</v>
-      </c>
-      <c r="F347" s="3" t="n">
-        <v>-266.86</v>
-      </c>
     </row>
     <row r="348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A348" s="3" t="n">
@@ -15040,42 +14164,6 @@
       <c r="B348" s="3" t="n">
         <v>-189.63</v>
       </c>
-      <c r="E348" s="3" t="n">
-        <v>398.65</v>
-      </c>
-      <c r="F348" s="3" t="n">
-        <v>-269.9</v>
-      </c>
-    </row>
-    <row r="349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A349" s="0"/>
-      <c r="B349" s="0"/>
-      <c r="E349" s="3" t="n">
-        <v>396.35</v>
-      </c>
-      <c r="F349" s="3" t="n">
-        <v>-273</v>
-      </c>
-    </row>
-    <row r="350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A350" s="0"/>
-      <c r="B350" s="0"/>
-      <c r="E350" s="3" t="n">
-        <v>393.46</v>
-      </c>
-      <c r="F350" s="3" t="n">
-        <v>-276.27</v>
-      </c>
-    </row>
-    <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A351" s="0"/>
-      <c r="B351" s="0"/>
-      <c r="E351" s="3" t="n">
-        <v>390.92</v>
-      </c>
-      <c r="F351" s="3" t="n">
-        <v>-276.94</v>
-      </c>
     </row>
     <row r="352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A352" s="1" t="s">
@@ -15084,12 +14172,6 @@
       <c r="B352" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E352" s="3" t="n">
-        <v>392.68</v>
-      </c>
-      <c r="F352" s="3" t="n">
-        <v>-273.18</v>
-      </c>
     </row>
     <row r="353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A353" s="1" t="s">
@@ -15098,12 +14180,6 @@
       <c r="B353" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E353" s="3" t="n">
-        <v>395.22</v>
-      </c>
-      <c r="F353" s="3" t="n">
-        <v>-269.43</v>
-      </c>
     </row>
     <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A354" s="1" t="s">
@@ -15112,12 +14188,6 @@
       <c r="B354" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E354" s="3" t="n">
-        <v>397.98</v>
-      </c>
-      <c r="F354" s="3" t="n">
-        <v>-265.13</v>
-      </c>
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A355" s="1" t="s">
@@ -15126,12 +14196,6 @@
       <c r="B355" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E355" s="3" t="n">
-        <v>398.86</v>
-      </c>
-      <c r="F355" s="3" t="n">
-        <v>-261.27</v>
-      </c>
     </row>
     <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="1" t="s">
@@ -15140,12 +14204,6 @@
       <c r="B356" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E356" s="3" t="n">
-        <v>398.97</v>
-      </c>
-      <c r="F356" s="3" t="n">
-        <v>-256.74</v>
-      </c>
     </row>
     <row r="357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="3" t="n">
@@ -15154,12 +14212,6 @@
       <c r="B357" s="3" t="n">
         <v>-223.51</v>
       </c>
-      <c r="E357" s="3" t="n">
-        <v>398.75</v>
-      </c>
-      <c r="F357" s="3" t="n">
-        <v>-252.66</v>
-      </c>
     </row>
     <row r="358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="3" t="n">
@@ -15168,12 +14220,6 @@
       <c r="B358" s="3" t="n">
         <v>-231.17</v>
       </c>
-      <c r="E358" s="3" t="n">
-        <v>397.43</v>
-      </c>
-      <c r="F358" s="3" t="n">
-        <v>-247.59</v>
-      </c>
     </row>
     <row r="359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="3" t="n">
@@ -15182,12 +14228,6 @@
       <c r="B359" s="3" t="n">
         <v>-237.04</v>
       </c>
-      <c r="E359" s="3" t="n">
-        <v>395.99</v>
-      </c>
-      <c r="F359" s="3" t="n">
-        <v>-243.28</v>
-      </c>
     </row>
     <row r="360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A360" s="12" t="n">
@@ -15196,12 +14236,6 @@
       <c r="B360" s="12" t="n">
         <v>-243.42</v>
       </c>
-      <c r="E360" s="3" t="n">
-        <v>394.45</v>
-      </c>
-      <c r="F360" s="3" t="n">
-        <v>-238.98</v>
-      </c>
     </row>
     <row r="361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="12" t="n">
@@ -15210,12 +14244,6 @@
       <c r="B361" s="12" t="n">
         <v>-247.05</v>
       </c>
-      <c r="E361" s="3" t="n">
-        <v>392.46</v>
-      </c>
-      <c r="F361" s="3" t="n">
-        <v>-235.89</v>
-      </c>
     </row>
     <row r="362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A362" s="3" t="n">
@@ -15224,12 +14252,6 @@
       <c r="B362" s="3" t="n">
         <v>-247.59</v>
       </c>
-      <c r="E362" s="3" t="n">
-        <v>389.37</v>
-      </c>
-      <c r="F362" s="3" t="n">
-        <v>-232.69</v>
-      </c>
     </row>
     <row r="363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="3" t="n">
@@ -15238,12 +14260,6 @@
       <c r="B363" s="3" t="n">
         <v>-243.28</v>
       </c>
-      <c r="E363" s="3" t="n">
-        <v>387.34</v>
-      </c>
-      <c r="F363" s="3" t="n">
-        <v>-228.28</v>
-      </c>
     </row>
     <row r="364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="3" t="n">
@@ -15252,12 +14268,6 @@
       <c r="B364" s="3" t="n">
         <v>-238.98</v>
       </c>
-      <c r="E364" s="3" t="n">
-        <v>384.79</v>
-      </c>
-      <c r="F364" s="3" t="n">
-        <v>-224.92</v>
-      </c>
     </row>
     <row r="365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="3" t="n">
@@ -15266,12 +14276,6 @@
       <c r="B365" s="3" t="n">
         <v>-235.89</v>
       </c>
-      <c r="E365" s="3" t="n">
-        <v>381.03</v>
-      </c>
-      <c r="F365" s="3" t="n">
-        <v>-221.97</v>
-      </c>
     </row>
     <row r="366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A366" s="3" t="n">
@@ -15280,39 +14284,21 @@
       <c r="B366" s="3" t="n">
         <v>-232.69</v>
       </c>
-      <c r="E366" s="3" t="n">
-        <v>377</v>
-      </c>
-      <c r="F366" s="3" t="n">
-        <v>-219.15</v>
-      </c>
     </row>
     <row r="367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A367" s="0" t="n">
+      <c r="A367" s="12" t="n">
         <v>387.34</v>
       </c>
-      <c r="B367" s="0" t="n">
+      <c r="B367" s="12" t="n">
         <v>-228.28</v>
       </c>
-      <c r="E367" s="3" t="n">
-        <v>374.58</v>
-      </c>
-      <c r="F367" s="3" t="n">
-        <v>-217.27</v>
-      </c>
     </row>
     <row r="368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A368" s="0" t="n">
+      <c r="A368" s="12" t="n">
         <v>384.79</v>
       </c>
-      <c r="B368" s="0" t="n">
+      <c r="B368" s="12" t="n">
         <v>-224.92</v>
-      </c>
-      <c r="E368" s="3" t="n">
-        <v>372.16</v>
-      </c>
-      <c r="F368" s="3" t="n">
-        <v>-214.98</v>
       </c>
     </row>
     <row r="369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15322,262 +14308,1944 @@
       <c r="B369" s="3" t="n">
         <v>-223.51</v>
       </c>
-      <c r="E369" s="3" t="n">
-        <v>368.94</v>
-      </c>
-      <c r="F369" s="3" t="n">
-        <v>-211.9</v>
-      </c>
     </row>
     <row r="370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A370" s="0"/>
       <c r="B370" s="0"/>
-      <c r="C370" s="3"/>
-      <c r="D370" s="3"/>
-      <c r="E370" s="3" t="n">
-        <v>364.64</v>
-      </c>
-      <c r="F370" s="3" t="n">
-        <v>-208.4</v>
+      <c r="C370" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D370" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="0"/>
       <c r="B371" s="0"/>
-      <c r="C371" s="3"/>
-      <c r="D371" s="3"/>
-      <c r="E371" s="3" t="n">
-        <v>359.01</v>
-      </c>
-      <c r="F371" s="3" t="n">
-        <v>-202.36</v>
+      <c r="C371" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D371" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="0"/>
       <c r="B372" s="0"/>
-      <c r="C372" s="3"/>
-      <c r="D372" s="3"/>
-      <c r="E372" s="3" t="n">
-        <v>353.23</v>
-      </c>
-      <c r="F372" s="3" t="n">
-        <v>-194.98</v>
+      <c r="C372" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D372" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="0"/>
       <c r="B373" s="0"/>
-      <c r="C373" s="3"/>
-      <c r="D373" s="3"/>
-      <c r="E373" s="3" t="n">
-        <v>344.5</v>
-      </c>
-      <c r="F373" s="3" t="n">
-        <v>-181.41</v>
+      <c r="C373" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D373" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="0"/>
       <c r="B374" s="0"/>
-      <c r="C374" s="3"/>
-      <c r="D374" s="3"/>
-      <c r="E374" s="3" t="n">
-        <v>340.18</v>
-      </c>
-      <c r="F374" s="3" t="n">
-        <v>-168.14</v>
+      <c r="C374" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D374" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="0"/>
       <c r="B375" s="0"/>
-      <c r="C375" s="3"/>
-      <c r="D375" s="3"/>
-      <c r="E375" s="3" t="n">
-        <v>338.64</v>
-      </c>
-      <c r="F375" s="3" t="n">
-        <v>-163.14</v>
+      <c r="C375" s="3" t="n">
+        <v>335.13</v>
+      </c>
+      <c r="D375" s="3" t="n">
+        <v>-320.95</v>
       </c>
     </row>
     <row r="376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="0"/>
       <c r="B376" s="0"/>
-      <c r="C376" s="3"/>
-      <c r="D376" s="3"/>
-      <c r="E376" s="3" t="n">
-        <v>336.66</v>
-      </c>
-      <c r="F376" s="3" t="n">
-        <v>-154.31</v>
+      <c r="C376" s="3" t="n">
+        <v>327.81</v>
+      </c>
+      <c r="D376" s="3" t="n">
+        <v>-316.94</v>
       </c>
     </row>
     <row r="377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="0"/>
       <c r="B377" s="0"/>
-      <c r="C377" s="3"/>
-      <c r="D377" s="3"/>
-      <c r="E377" s="3" t="n">
-        <v>334.72</v>
-      </c>
-      <c r="F377" s="3" t="n">
-        <v>-161.55</v>
+      <c r="C377" s="3" t="n">
+        <v>320.49</v>
+      </c>
+      <c r="D377" s="3" t="n">
+        <v>-310.1</v>
       </c>
     </row>
     <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="0"/>
       <c r="B378" s="0"/>
-      <c r="C378" s="3"/>
-      <c r="D378" s="3"/>
-      <c r="E378" s="3" t="n">
+      <c r="C378" s="3" t="n">
+        <v>315.54</v>
+      </c>
+      <c r="D378" s="3" t="n">
+        <v>-301.83</v>
+      </c>
+    </row>
+    <row r="379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A379" s="0"/>
+      <c r="B379" s="0"/>
+      <c r="C379" s="3" t="n">
+        <v>309.4</v>
+      </c>
+      <c r="D379" s="3" t="n">
+        <v>-291.45</v>
+      </c>
+    </row>
+    <row r="380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A380" s="0"/>
+      <c r="B380" s="0"/>
+      <c r="C380" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="D380" s="3" t="n">
+        <v>-280</v>
+      </c>
+    </row>
+    <row r="381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A381" s="0"/>
+      <c r="B381" s="0"/>
+      <c r="C381" s="3" t="n">
+        <v>294.53</v>
+      </c>
+      <c r="D381" s="3" t="n">
+        <v>-271.62</v>
+      </c>
+    </row>
+    <row r="382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A382" s="0"/>
+      <c r="B382" s="0"/>
+      <c r="C382" s="3" t="n">
+        <v>300.43</v>
+      </c>
+      <c r="D382" s="3" t="n">
+        <v>-286.49</v>
+      </c>
+    </row>
+    <row r="383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A383" s="0"/>
+      <c r="B383" s="0"/>
+      <c r="C383" s="3" t="n">
+        <v>294.29</v>
+      </c>
+      <c r="D383" s="3" t="n">
+        <v>-285.78</v>
+      </c>
+    </row>
+    <row r="384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A384" s="0"/>
+      <c r="B384" s="0"/>
+      <c r="C384" s="3" t="n">
+        <v>293.58</v>
+      </c>
+      <c r="D384" s="3" t="n">
+        <v>-281.77</v>
+      </c>
+    </row>
+    <row r="385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A385" s="0"/>
+      <c r="B385" s="0"/>
+      <c r="C385" s="3" t="n">
+        <v>287.45</v>
+      </c>
+      <c r="D385" s="3" t="n">
+        <v>-273.98</v>
+      </c>
+    </row>
+    <row r="386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A386" s="0"/>
+      <c r="B386" s="0"/>
+      <c r="C386" s="3" t="n">
+        <v>283.2</v>
+      </c>
+      <c r="D386" s="3" t="n">
+        <v>-268.08</v>
+      </c>
+    </row>
+    <row r="387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A387" s="0"/>
+      <c r="B387" s="0"/>
+      <c r="C387" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="D387" s="3" t="n">
+        <v>-260</v>
+      </c>
+    </row>
+    <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A388" s="0"/>
+      <c r="B388" s="0"/>
+      <c r="C388" s="3" t="n">
+        <v>274.23</v>
+      </c>
+      <c r="D388" s="3" t="n">
+        <v>-249.2</v>
+      </c>
+    </row>
+    <row r="389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A389" s="0"/>
+      <c r="B389" s="0"/>
+      <c r="C389" s="3" t="n">
+        <v>270.69</v>
+      </c>
+      <c r="D389" s="3" t="n">
+        <v>-237.16</v>
+      </c>
+    </row>
+    <row r="390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A390" s="0"/>
+      <c r="B390" s="0"/>
+      <c r="C390" s="3" t="n">
+        <v>268.56</v>
+      </c>
+      <c r="D390" s="3" t="n">
+        <v>-232.2</v>
+      </c>
+    </row>
+    <row r="391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A391" s="0"/>
+      <c r="B391" s="0"/>
+      <c r="C391" s="3" t="n">
+        <v>267.62</v>
+      </c>
+      <c r="D391" s="3" t="n">
+        <v>-240.7</v>
+      </c>
+    </row>
+    <row r="392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A392" s="0"/>
+      <c r="B392" s="0"/>
+      <c r="C392" s="3" t="n">
+        <v>268.56</v>
+      </c>
+      <c r="D392" s="3" t="n">
+        <v>-247.07</v>
+      </c>
+    </row>
+    <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A393" s="0"/>
+      <c r="B393" s="0"/>
+      <c r="C393" s="3" t="n">
+        <v>270.45</v>
+      </c>
+      <c r="D393" s="3" t="n">
+        <v>-254.15</v>
+      </c>
+    </row>
+    <row r="394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A394" s="0"/>
+      <c r="B394" s="0"/>
+      <c r="C394" s="3" t="n">
+        <v>273.99</v>
+      </c>
+      <c r="D394" s="3" t="n">
+        <v>-259.82</v>
+      </c>
+    </row>
+    <row r="395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A395" s="0"/>
+      <c r="B395" s="0"/>
+      <c r="C395" s="3" t="n">
+        <v>276.12</v>
+      </c>
+      <c r="D395" s="3" t="n">
+        <v>-264.3</v>
+      </c>
+    </row>
+    <row r="396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A396" s="0"/>
+      <c r="B396" s="0"/>
+      <c r="C396" s="3" t="n">
+        <v>270.45</v>
+      </c>
+      <c r="D396" s="3" t="n">
+        <v>-261.47</v>
+      </c>
+    </row>
+    <row r="397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A397" s="0"/>
+      <c r="B397" s="0"/>
+      <c r="C397" s="3" t="n">
+        <v>265.97</v>
+      </c>
+      <c r="D397" s="3" t="n">
+        <v>-255.57</v>
+      </c>
+    </row>
+    <row r="398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A398" s="0"/>
+      <c r="B398" s="0"/>
+      <c r="C398" s="3" t="n">
+        <v>262.43</v>
+      </c>
+      <c r="D398" s="3" t="n">
+        <v>-249.2</v>
+      </c>
+    </row>
+    <row r="399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A399" s="0"/>
+      <c r="B399" s="0"/>
+      <c r="C399" s="3" t="n">
+        <v>260</v>
+      </c>
+      <c r="D399" s="3" t="n">
+        <v>-240</v>
+      </c>
+    </row>
+    <row r="400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A400" s="0"/>
+      <c r="B400" s="0"/>
+      <c r="C400" s="3" t="n">
+        <v>260.77</v>
+      </c>
+      <c r="D400" s="3" t="n">
+        <v>-227.95</v>
+      </c>
+    </row>
+    <row r="401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A401" s="0"/>
+      <c r="B401" s="0"/>
+      <c r="C401" s="3" t="n">
+        <v>267.48</v>
+      </c>
+      <c r="D401" s="3" t="n">
+        <v>-169.91</v>
+      </c>
+    </row>
+    <row r="402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A402" s="0"/>
+      <c r="B402" s="0"/>
+      <c r="C402" s="3" t="n">
+        <v>273.14</v>
+      </c>
+      <c r="D402" s="3" t="n">
+        <v>-151.69</v>
+      </c>
+    </row>
+    <row r="403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A403" s="0"/>
+      <c r="B403" s="0"/>
+      <c r="C403" s="3" t="n">
+        <v>281.84</v>
+      </c>
+      <c r="D403" s="3" t="n">
+        <v>-136.34</v>
+      </c>
+    </row>
+    <row r="404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A404" s="0"/>
+      <c r="B404" s="0"/>
+      <c r="C404" s="3" t="n">
+        <v>292.95</v>
+      </c>
+      <c r="D404" s="3" t="n">
+        <v>-120.55</v>
+      </c>
+    </row>
+    <row r="405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A405" s="0"/>
+      <c r="B405" s="0"/>
+      <c r="C405" s="3" t="n">
+        <v>304.8</v>
+      </c>
+      <c r="D405" s="3" t="n">
+        <v>-108.2</v>
+      </c>
+    </row>
+    <row r="406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A406" s="0"/>
+      <c r="B406" s="0"/>
+      <c r="C406" s="3" t="n">
+        <v>316.63</v>
+      </c>
+      <c r="D406" s="3" t="n">
+        <v>-99.15</v>
+      </c>
+    </row>
+    <row r="407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A407" s="0"/>
+      <c r="B407" s="0"/>
+      <c r="C407" s="3" t="n">
+        <v>329.06</v>
+      </c>
+      <c r="D407" s="3" t="n">
+        <v>-92.94</v>
+      </c>
+    </row>
+    <row r="408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A408" s="0"/>
+      <c r="B408" s="0"/>
+      <c r="C408" s="3" t="n">
+        <v>343.56</v>
+      </c>
+      <c r="D408" s="3" t="n">
+        <v>-92.52</v>
+      </c>
+    </row>
+    <row r="409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A409" s="0"/>
+      <c r="B409" s="0"/>
+      <c r="C409" s="3" t="n">
+        <v>355.99</v>
+      </c>
+      <c r="D409" s="3" t="n">
+        <v>-86.72</v>
+      </c>
+    </row>
+    <row r="410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A410" s="0"/>
+      <c r="B410" s="0"/>
+      <c r="C410" s="3" t="n">
+        <v>368.01</v>
+      </c>
+      <c r="D410" s="3" t="n">
+        <v>-87.14</v>
+      </c>
+    </row>
+    <row r="411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A411" s="0"/>
+      <c r="B411" s="0"/>
+      <c r="C411" s="3" t="n">
+        <v>380.03</v>
+      </c>
+      <c r="D411" s="3" t="n">
+        <v>-88.79</v>
+      </c>
+    </row>
+    <row r="412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A412" s="0"/>
+      <c r="B412" s="0"/>
+      <c r="C412" s="3" t="n">
+        <v>391.63</v>
+      </c>
+      <c r="D412" s="3" t="n">
+        <v>-91.28</v>
+      </c>
+    </row>
+    <row r="413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A413" s="0"/>
+      <c r="B413" s="0"/>
+      <c r="C413" s="3" t="n">
+        <v>403.23</v>
+      </c>
+      <c r="D413" s="3" t="n">
+        <v>-95.84</v>
+      </c>
+    </row>
+    <row r="414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A414" s="0"/>
+      <c r="B414" s="0"/>
+      <c r="C414" s="3" t="n">
+        <v>412.76</v>
+      </c>
+      <c r="D414" s="3" t="n">
+        <v>-101.22</v>
+      </c>
+    </row>
+    <row r="415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A415" s="0"/>
+      <c r="B415" s="0"/>
+      <c r="C415" s="3" t="n">
+        <v>424.36</v>
+      </c>
+      <c r="D415" s="3" t="n">
+        <v>-107.85</v>
+      </c>
+    </row>
+    <row r="416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A416" s="0"/>
+      <c r="B416" s="0"/>
+      <c r="C416" s="3" t="n">
+        <v>432.23</v>
+      </c>
+      <c r="D416" s="3" t="n">
+        <v>-113.24</v>
+      </c>
+    </row>
+    <row r="417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A417" s="0"/>
+      <c r="B417" s="0"/>
+      <c r="C417" s="3" t="n">
+        <v>443.01</v>
+      </c>
+      <c r="D417" s="3" t="n">
+        <v>-122.35</v>
+      </c>
+    </row>
+    <row r="418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A418" s="0"/>
+      <c r="B418" s="0"/>
+      <c r="C418" s="3" t="n">
+        <v>450.88</v>
+      </c>
+      <c r="D418" s="3" t="n">
+        <v>-131.47</v>
+      </c>
+    </row>
+    <row r="419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A419" s="0"/>
+      <c r="B419" s="0"/>
+      <c r="C419" s="3" t="n">
+        <v>455.44</v>
+      </c>
+      <c r="D419" s="3" t="n">
+        <v>-137.69</v>
+      </c>
+    </row>
+    <row r="420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A420" s="0"/>
+      <c r="B420" s="0"/>
+      <c r="C420" s="3" t="n">
+        <v>461.65</v>
+      </c>
+      <c r="D420" s="3" t="n">
+        <v>-146.39</v>
+      </c>
+    </row>
+    <row r="421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A421" s="0"/>
+      <c r="B421" s="0"/>
+      <c r="C421" s="3" t="n">
+        <v>468.28</v>
+      </c>
+      <c r="D421" s="3" t="n">
+        <v>-158.4</v>
+      </c>
+    </row>
+    <row r="422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A422" s="0"/>
+      <c r="B422" s="0"/>
+      <c r="C422" s="3" t="n">
+        <v>470.77</v>
+      </c>
+      <c r="D422" s="3" t="n">
+        <v>-170.42</v>
+      </c>
+    </row>
+    <row r="423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A423" s="0"/>
+      <c r="B423" s="0"/>
+      <c r="C423" s="3" t="n">
+        <v>474.08</v>
+      </c>
+      <c r="D423" s="3" t="n">
+        <v>-180.36</v>
+      </c>
+    </row>
+    <row r="424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A424" s="0"/>
+      <c r="B424" s="0"/>
+      <c r="C424" s="3" t="n">
+        <v>477.4</v>
+      </c>
+      <c r="D424" s="3" t="n">
+        <v>-191.14</v>
+      </c>
+    </row>
+    <row r="425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A425" s="0"/>
+      <c r="B425" s="0"/>
+      <c r="C425" s="3" t="n">
+        <v>476.98</v>
+      </c>
+      <c r="D425" s="3" t="n">
+        <v>-201.08</v>
+      </c>
+    </row>
+    <row r="426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A426" s="0"/>
+      <c r="B426" s="0"/>
+      <c r="C426" s="3" t="n">
+        <v>477.4</v>
+      </c>
+      <c r="D426" s="3" t="n">
+        <v>-211.44</v>
+      </c>
+    </row>
+    <row r="427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A427" s="0"/>
+      <c r="B427" s="0"/>
+      <c r="C427" s="3" t="n">
+        <v>480</v>
+      </c>
+      <c r="D427" s="3" t="n">
+        <v>-220</v>
+      </c>
+    </row>
+    <row r="428" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A428" s="0"/>
+      <c r="B428" s="0"/>
+      <c r="C428" s="3" t="n">
+        <v>478.64</v>
+      </c>
+      <c r="D428" s="3" t="n">
+        <v>-230.5</v>
+      </c>
+    </row>
+    <row r="429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A429" s="0"/>
+      <c r="B429" s="0"/>
+      <c r="C429" s="3" t="n">
+        <v>477.4</v>
+      </c>
+      <c r="D429" s="3" t="n">
+        <v>-241.69</v>
+      </c>
+    </row>
+    <row r="430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A430" s="0"/>
+      <c r="B430" s="0"/>
+      <c r="C430" s="3" t="n">
+        <v>476.98</v>
+      </c>
+      <c r="D430" s="3" t="n">
+        <v>-252.46</v>
+      </c>
+    </row>
+    <row r="431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A431" s="0"/>
+      <c r="B431" s="0"/>
+      <c r="C431" s="3" t="n">
+        <v>473.67</v>
+      </c>
+      <c r="D431" s="3" t="n">
+        <v>-262.4</v>
+      </c>
+    </row>
+    <row r="432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A432" s="0"/>
+      <c r="B432" s="0"/>
+      <c r="C432" s="3" t="n">
+        <v>470.35</v>
+      </c>
+      <c r="D432" s="3" t="n">
+        <v>-271.52</v>
+      </c>
+    </row>
+    <row r="433" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A433" s="0"/>
+      <c r="B433" s="0"/>
+      <c r="C433" s="3" t="n">
+        <v>466.21</v>
+      </c>
+      <c r="D433" s="3" t="n">
+        <v>-281.88</v>
+      </c>
+    </row>
+    <row r="434" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A434" s="0"/>
+      <c r="B434" s="0"/>
+      <c r="C434" s="3" t="n">
+        <v>470.28</v>
+      </c>
+      <c r="D434" s="3" t="n">
+        <v>-266.73</v>
+      </c>
+    </row>
+    <row r="435" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A435" s="0"/>
+      <c r="B435" s="0"/>
+      <c r="C435" s="3" t="n">
+        <v>471.83</v>
+      </c>
+      <c r="D435" s="3" t="n">
+        <v>-258.69</v>
+      </c>
+    </row>
+    <row r="436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A436" s="0"/>
+      <c r="B436" s="0"/>
+      <c r="C436" s="3" t="n">
+        <v>472.11</v>
+      </c>
+      <c r="D436" s="3" t="n">
+        <v>-249.66</v>
+      </c>
+    </row>
+    <row r="437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A437" s="0"/>
+      <c r="B437" s="0"/>
+      <c r="C437" s="3" t="n">
+        <v>472.39</v>
+      </c>
+      <c r="D437" s="3" t="n">
+        <v>-240.62</v>
+      </c>
+    </row>
+    <row r="438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A438" s="0"/>
+      <c r="B438" s="0"/>
+      <c r="C438" s="3" t="n">
+        <v>472.96</v>
+      </c>
+      <c r="D438" s="3" t="n">
+        <v>-232.16</v>
+      </c>
+    </row>
+    <row r="439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A439" s="0"/>
+      <c r="B439" s="0"/>
+      <c r="C439" s="3" t="n">
+        <v>470.98</v>
+      </c>
+      <c r="D439" s="3" t="n">
+        <v>-223.97</v>
+      </c>
+    </row>
+    <row r="440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A440" s="0"/>
+      <c r="B440" s="0"/>
+      <c r="C440" s="3" t="n">
+        <v>469.99</v>
+      </c>
+      <c r="D440" s="3" t="n">
+        <v>-216.63</v>
+      </c>
+    </row>
+    <row r="441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A441" s="0"/>
+      <c r="B441" s="0"/>
+      <c r="C441" s="3" t="n">
+        <v>467.45</v>
+      </c>
+      <c r="D441" s="3" t="n">
+        <v>-209.29</v>
+      </c>
+    </row>
+    <row r="442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A442" s="0"/>
+      <c r="B442" s="0"/>
+      <c r="C442" s="3" t="n">
+        <v>465.76</v>
+      </c>
+      <c r="D442" s="3" t="n">
+        <v>-214.37</v>
+      </c>
+    </row>
+    <row r="443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A443" s="0"/>
+      <c r="B443" s="0"/>
+      <c r="C443" s="3" t="n">
+        <v>466.18</v>
+      </c>
+      <c r="D443" s="3" t="n">
+        <v>-221.71</v>
+      </c>
+    </row>
+    <row r="444" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A444" s="0"/>
+      <c r="B444" s="0"/>
+      <c r="C444" s="3" t="n">
+        <v>465.62</v>
+      </c>
+      <c r="D444" s="3" t="n">
+        <v>-228.2</v>
+      </c>
+    </row>
+    <row r="445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A445" s="0"/>
+      <c r="B445" s="0"/>
+      <c r="C445" s="3" t="n">
+        <v>464.21</v>
+      </c>
+      <c r="D445" s="3" t="n">
+        <v>-234.13</v>
+      </c>
+    </row>
+    <row r="446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A446" s="0"/>
+      <c r="B446" s="0"/>
+      <c r="C446" s="3" t="n">
+        <v>463.36</v>
+      </c>
+      <c r="D446" s="3" t="n">
+        <v>-239.21</v>
+      </c>
+    </row>
+    <row r="447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A447" s="0"/>
+      <c r="B447" s="0"/>
+      <c r="C447" s="3" t="n">
+        <v>462.09</v>
+      </c>
+      <c r="D447" s="3" t="n">
+        <v>-244.86</v>
+      </c>
+    </row>
+    <row r="448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A448" s="0"/>
+      <c r="B448" s="0"/>
+      <c r="C448" s="3" t="n">
+        <v>460.4</v>
+      </c>
+      <c r="D448" s="3" t="n">
+        <v>-248.67</v>
+      </c>
+    </row>
+    <row r="449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A449" s="0"/>
+      <c r="B449" s="0"/>
+      <c r="C449" s="3" t="n">
+        <v>458.42</v>
+      </c>
+      <c r="D449" s="3" t="n">
+        <v>-253.04</v>
+      </c>
+    </row>
+    <row r="450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A450" s="0"/>
+      <c r="B450" s="0"/>
+      <c r="C450" s="3" t="n">
+        <v>456.59</v>
+      </c>
+      <c r="D450" s="3" t="n">
+        <v>-257.42</v>
+      </c>
+    </row>
+    <row r="451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A451" s="0"/>
+      <c r="B451" s="0"/>
+      <c r="C451" s="3" t="n">
+        <v>454.05</v>
+      </c>
+      <c r="D451" s="3" t="n">
+        <v>-262.08</v>
+      </c>
+    </row>
+    <row r="452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A452" s="0"/>
+      <c r="B452" s="0"/>
+      <c r="C452" s="3" t="n">
+        <v>450.94</v>
+      </c>
+      <c r="D452" s="3" t="n">
+        <v>-267.72</v>
+      </c>
+    </row>
+    <row r="453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A453" s="0"/>
+      <c r="B453" s="0"/>
+      <c r="C453" s="3" t="n">
+        <v>449.36</v>
+      </c>
+      <c r="D453" s="3" t="n">
+        <v>-273.26</v>
+      </c>
+    </row>
+    <row r="454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A454" s="0"/>
+      <c r="B454" s="0"/>
+      <c r="C454" s="3" t="n">
+        <v>451.22</v>
+      </c>
+      <c r="D454" s="3" t="n">
+        <v>-279.88</v>
+      </c>
+    </row>
+    <row r="455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A455" s="0"/>
+      <c r="B455" s="0"/>
+      <c r="C455" s="3" t="n">
+        <v>453.91</v>
+      </c>
+      <c r="D455" s="3" t="n">
+        <v>-286.7</v>
+      </c>
+    </row>
+    <row r="456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A456" s="0"/>
+      <c r="B456" s="0"/>
+      <c r="C456" s="3" t="n">
+        <v>455.11</v>
+      </c>
+      <c r="D456" s="3" t="n">
+        <v>-292.87</v>
+      </c>
+    </row>
+    <row r="457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A457" s="0"/>
+      <c r="B457" s="0"/>
+      <c r="C457" s="3" t="n">
+        <v>457.77</v>
+      </c>
+      <c r="D457" s="3" t="n">
+        <v>-296.86</v>
+      </c>
+    </row>
+    <row r="458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A458" s="0"/>
+      <c r="B458" s="0"/>
+      <c r="C458" s="3" t="n">
+        <v>451.57</v>
+      </c>
+      <c r="D458" s="3" t="n">
+        <v>-291.99</v>
+      </c>
+    </row>
+    <row r="459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A459" s="0"/>
+      <c r="B459" s="0"/>
+      <c r="C459" s="3" t="n">
+        <v>448.24</v>
+      </c>
+      <c r="D459" s="3" t="n">
+        <v>-286.23</v>
+      </c>
+    </row>
+    <row r="460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A460" s="0"/>
+      <c r="B460" s="0"/>
+      <c r="C460" s="3" t="n">
+        <v>445.14</v>
+      </c>
+      <c r="D460" s="3" t="n">
+        <v>-276.7</v>
+      </c>
+    </row>
+    <row r="461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A461" s="0"/>
+      <c r="B461" s="0"/>
+      <c r="C461" s="3" t="n">
+        <v>442.49</v>
+      </c>
+      <c r="D461" s="3" t="n">
+        <v>-272.05</v>
+      </c>
+    </row>
+    <row r="462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A462" s="0"/>
+      <c r="B462" s="0"/>
+      <c r="C462" s="3" t="n">
+        <v>440</v>
+      </c>
+      <c r="D462" s="3" t="n">
+        <v>-280</v>
+      </c>
+    </row>
+    <row r="463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A463" s="0"/>
+      <c r="B463" s="0"/>
+      <c r="C463" s="3" t="n">
+        <v>437.66</v>
+      </c>
+      <c r="D463" s="3" t="n">
+        <v>-287.08</v>
+      </c>
+    </row>
+    <row r="464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A464" s="0"/>
+      <c r="B464" s="0"/>
+      <c r="C464" s="3" t="n">
+        <v>433.77</v>
+      </c>
+      <c r="D464" s="3" t="n">
+        <v>-293.89</v>
+      </c>
+    </row>
+    <row r="465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A465" s="0"/>
+      <c r="B465" s="0"/>
+      <c r="C465" s="3" t="n">
+        <v>429.88</v>
+      </c>
+      <c r="D465" s="3" t="n">
+        <v>-300.7</v>
+      </c>
+    </row>
+    <row r="466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A466" s="0"/>
+      <c r="B466" s="0"/>
+      <c r="C466" s="3" t="n">
+        <v>425.99</v>
+      </c>
+      <c r="D466" s="3" t="n">
+        <v>-306.54</v>
+      </c>
+    </row>
+    <row r="467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A467" s="0"/>
+      <c r="B467" s="0"/>
+      <c r="C467" s="3" t="n">
+        <v>422.73</v>
+      </c>
+      <c r="D467" s="3" t="n">
+        <v>-310.62</v>
+      </c>
+    </row>
+    <row r="468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A468" s="0"/>
+      <c r="B468" s="0"/>
+      <c r="C468" s="3" t="n">
+        <v>420.02</v>
+      </c>
+      <c r="D468" s="3" t="n">
+        <v>-314.11</v>
+      </c>
+    </row>
+    <row r="469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A469" s="0"/>
+      <c r="B469" s="0"/>
+      <c r="C469" s="3" t="n">
+        <v>417.04</v>
+      </c>
+      <c r="D469" s="3" t="n">
+        <v>-317.6</v>
+      </c>
+    </row>
+    <row r="470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A470" s="0"/>
+      <c r="B470" s="0"/>
+      <c r="C470" s="3" t="n">
+        <v>409.67</v>
+      </c>
+      <c r="D470" s="3" t="n">
+        <v>-323.42</v>
+      </c>
+    </row>
+    <row r="471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A471" s="0"/>
+      <c r="B471" s="0"/>
+      <c r="C471" s="3" t="n">
+        <v>406.31</v>
+      </c>
+      <c r="D471" s="3" t="n">
+        <v>-325.36</v>
+      </c>
+    </row>
+    <row r="472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A472" s="0"/>
+      <c r="B472" s="0"/>
+      <c r="C472" s="3" t="n">
+        <v>410</v>
+      </c>
+      <c r="D472" s="3" t="n">
+        <v>-320</v>
+      </c>
+    </row>
+    <row r="473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A473" s="0"/>
+      <c r="B473" s="0"/>
+      <c r="C473" s="3" t="n">
+        <v>413.55</v>
+      </c>
+      <c r="D473" s="3" t="n">
+        <v>-313.85</v>
+      </c>
+    </row>
+    <row r="474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A474" s="0"/>
+      <c r="B474" s="0"/>
+      <c r="C474" s="3" t="n">
+        <v>416.91</v>
+      </c>
+      <c r="D474" s="3" t="n">
+        <v>-308.29</v>
+      </c>
+    </row>
+    <row r="475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A475" s="0"/>
+      <c r="B475" s="0"/>
+      <c r="C475" s="3" t="n">
+        <v>420.53</v>
+      </c>
+      <c r="D475" s="3" t="n">
+        <v>-302.86</v>
+      </c>
+    </row>
+    <row r="476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A476" s="0"/>
+      <c r="B476" s="0"/>
+      <c r="C476" s="3" t="n">
+        <v>423.25</v>
+      </c>
+      <c r="D476" s="3" t="n">
+        <v>-296.78</v>
+      </c>
+    </row>
+    <row r="477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A477" s="0"/>
+      <c r="B477" s="0"/>
+      <c r="C477" s="3" t="n">
+        <v>426.48</v>
+      </c>
+      <c r="D477" s="3" t="n">
+        <v>-286.95</v>
+      </c>
+    </row>
+    <row r="478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A478" s="0"/>
+      <c r="B478" s="0"/>
+      <c r="C478" s="3" t="n">
+        <v>428.22</v>
+      </c>
+      <c r="D478" s="3" t="n">
+        <v>-279.6</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A479" s="0"/>
+      <c r="B479" s="0"/>
+      <c r="C479" s="3" t="n">
+        <v>429.77</v>
+      </c>
+      <c r="D479" s="3" t="n">
+        <v>-272.83</v>
+      </c>
+    </row>
+    <row r="480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A480" s="0"/>
+      <c r="B480" s="0"/>
+      <c r="C480" s="3" t="n">
+        <v>430.93</v>
+      </c>
+      <c r="D480" s="3" t="n">
+        <v>-264.12</v>
+      </c>
+    </row>
+    <row r="481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A481" s="0"/>
+      <c r="B481" s="0"/>
+      <c r="C481" s="3" t="n">
+        <v>430</v>
+      </c>
+      <c r="D481" s="3" t="n">
+        <v>-260</v>
+      </c>
+    </row>
+    <row r="482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A482" s="0"/>
+      <c r="B482" s="0"/>
+      <c r="C482" s="3" t="n">
+        <v>427.64</v>
+      </c>
+      <c r="D482" s="3" t="n">
+        <v>-267.6</v>
+      </c>
+    </row>
+    <row r="483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A483" s="0"/>
+      <c r="B483" s="0"/>
+      <c r="C483" s="3" t="n">
+        <v>424.16</v>
+      </c>
+      <c r="D483" s="3" t="n">
+        <v>-275.92</v>
+      </c>
+    </row>
+    <row r="484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A484" s="0"/>
+      <c r="B484" s="0"/>
+      <c r="C484" s="3" t="n">
+        <v>420.87</v>
+      </c>
+      <c r="D484" s="3" t="n">
+        <v>-282.31</v>
+      </c>
+    </row>
+    <row r="485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A485" s="0"/>
+      <c r="B485" s="0"/>
+      <c r="C485" s="3" t="n">
+        <v>418.74</v>
+      </c>
+      <c r="D485" s="3" t="n">
+        <v>-287.53</v>
+      </c>
+    </row>
+    <row r="486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A486" s="0"/>
+      <c r="B486" s="0"/>
+      <c r="C486" s="3" t="n">
+        <v>413.71</v>
+      </c>
+      <c r="D486" s="3" t="n">
+        <v>-293.92</v>
+      </c>
+    </row>
+    <row r="487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A487" s="0"/>
+      <c r="B487" s="0"/>
+      <c r="C487" s="3" t="n">
+        <v>420.04</v>
+      </c>
+      <c r="D487" s="3" t="n">
+        <v>-275.55</v>
+      </c>
+    </row>
+    <row r="488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A488" s="0"/>
+      <c r="B488" s="0"/>
+      <c r="C488" s="3" t="n">
+        <v>421.95</v>
+      </c>
+      <c r="D488" s="3" t="n">
+        <v>-264.91</v>
+      </c>
+    </row>
+    <row r="489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A489" s="0"/>
+      <c r="B489" s="0"/>
+      <c r="C489" s="3" t="n">
+        <v>424.73</v>
+      </c>
+      <c r="D489" s="3" t="n">
+        <v>-217.03</v>
+      </c>
+    </row>
+    <row r="490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A490" s="0"/>
+      <c r="B490" s="0"/>
+      <c r="C490" s="3" t="n">
+        <v>424.57</v>
+      </c>
+      <c r="D490" s="3" t="n">
+        <v>-210.38</v>
+      </c>
+    </row>
+    <row r="491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A491" s="0"/>
+      <c r="B491" s="0"/>
+      <c r="C491" s="3" t="n">
+        <v>409.81</v>
+      </c>
+      <c r="D491" s="3" t="n">
+        <v>-194.69</v>
+      </c>
+    </row>
+    <row r="492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A492" s="0"/>
+      <c r="B492" s="0"/>
+      <c r="C492" s="3" t="n">
+        <v>390.37</v>
+      </c>
+      <c r="D492" s="3" t="n">
+        <v>-167.38</v>
+      </c>
+    </row>
+    <row r="493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A493" s="0"/>
+      <c r="B493" s="0"/>
+      <c r="C493" s="3" t="n">
+        <v>389.68</v>
+      </c>
+      <c r="D493" s="3" t="n">
+        <v>-178.19</v>
+      </c>
+    </row>
+    <row r="494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A494" s="0"/>
+      <c r="B494" s="0"/>
+      <c r="C494" s="3" t="n">
+        <v>388.22</v>
+      </c>
+      <c r="D494" s="3" t="n">
+        <v>-189.63</v>
+      </c>
+    </row>
+    <row r="495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A495" s="0"/>
+      <c r="B495" s="0"/>
+      <c r="C495" s="3" t="n">
+        <v>390</v>
+      </c>
+      <c r="D495" s="3" t="n">
+        <v>-198.49</v>
+      </c>
+    </row>
+    <row r="496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A496" s="0"/>
+      <c r="B496" s="0"/>
+      <c r="C496" s="3" t="n">
+        <v>391.54</v>
+      </c>
+      <c r="D496" s="3" t="n">
+        <v>-206.15</v>
+      </c>
+    </row>
+    <row r="497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A497" s="0"/>
+      <c r="B497" s="0"/>
+      <c r="C497" s="3" t="n">
+        <v>393.32</v>
+      </c>
+      <c r="D497" s="3" t="n">
+        <v>-214.57</v>
+      </c>
+    </row>
+    <row r="498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A498" s="0"/>
+      <c r="B498" s="0"/>
+      <c r="C498" s="3" t="n">
+        <v>396.13</v>
+      </c>
+      <c r="D498" s="3" t="n">
+        <v>-223.51</v>
+      </c>
+    </row>
+    <row r="499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A499" s="0"/>
+      <c r="B499" s="0"/>
+      <c r="C499" s="3" t="n">
+        <v>400.21</v>
+      </c>
+      <c r="D499" s="3" t="n">
+        <v>-231.17</v>
+      </c>
+    </row>
+    <row r="500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A500" s="0"/>
+      <c r="B500" s="0"/>
+      <c r="C500" s="3" t="n">
+        <v>402.77</v>
+      </c>
+      <c r="D500" s="3" t="n">
+        <v>-237.04</v>
+      </c>
+    </row>
+    <row r="501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A501" s="0"/>
+      <c r="B501" s="0"/>
+      <c r="C501" s="3" t="n">
+        <v>406.6</v>
+      </c>
+      <c r="D501" s="3" t="n">
+        <v>-243.42</v>
+      </c>
+    </row>
+    <row r="502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A502" s="0"/>
+      <c r="B502" s="0"/>
+      <c r="C502" s="3" t="n">
+        <v>410.68</v>
+      </c>
+      <c r="D502" s="3" t="n">
+        <v>-246.74</v>
+      </c>
+    </row>
+    <row r="503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A503" s="0"/>
+      <c r="B503" s="0"/>
+      <c r="C503" s="3" t="n">
+        <v>412.33</v>
+      </c>
+      <c r="D503" s="3" t="n">
+        <v>-249.78</v>
+      </c>
+    </row>
+    <row r="504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A504" s="0"/>
+      <c r="B504" s="0"/>
+      <c r="C504" s="3" t="n">
+        <v>415</v>
+      </c>
+      <c r="D504" s="3" t="n">
+        <v>-250</v>
+      </c>
+    </row>
+    <row r="505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A505" s="0"/>
+      <c r="B505" s="0"/>
+      <c r="C505" s="3" t="n">
+        <v>411.07</v>
+      </c>
+      <c r="D505" s="3" t="n">
+        <v>-250.74</v>
+      </c>
+    </row>
+    <row r="506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A506" s="0"/>
+      <c r="B506" s="0"/>
+      <c r="C506" s="3" t="n">
+        <v>408.7</v>
+      </c>
+      <c r="D506" s="3" t="n">
+        <v>-249.27</v>
+      </c>
+    </row>
+    <row r="507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A507" s="0"/>
+      <c r="B507" s="0"/>
+      <c r="C507" s="3" t="n">
+        <v>406.56</v>
+      </c>
+      <c r="D507" s="3" t="n">
+        <v>-247.49</v>
+      </c>
+    </row>
+    <row r="508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A508" s="0"/>
+      <c r="B508" s="0"/>
+      <c r="C508" s="3" t="n">
+        <v>404.86</v>
+      </c>
+      <c r="D508" s="3" t="n">
+        <v>-247.05</v>
+      </c>
+    </row>
+    <row r="509" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A509" s="0"/>
+      <c r="B509" s="0"/>
+      <c r="C509" s="3" t="n">
+        <v>405</v>
+      </c>
+      <c r="D509" s="3" t="n">
+        <v>-250</v>
+      </c>
+    </row>
+    <row r="510" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A510" s="0"/>
+      <c r="B510" s="0"/>
+      <c r="C510" s="3" t="n">
+        <v>404.86</v>
+      </c>
+      <c r="D510" s="3" t="n">
+        <v>-252.74</v>
+      </c>
+    </row>
+    <row r="511" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A511" s="0"/>
+      <c r="B511" s="0"/>
+      <c r="C511" s="3" t="n">
+        <v>405</v>
+      </c>
+      <c r="D511" s="3" t="n">
+        <v>-255</v>
+      </c>
+    </row>
+    <row r="512" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A512" s="0"/>
+      <c r="B512" s="0"/>
+      <c r="C512" s="3" t="n">
+        <v>404.19</v>
+      </c>
+      <c r="D512" s="3" t="n">
+        <v>-258.58</v>
+      </c>
+    </row>
+    <row r="513" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A513" s="0"/>
+      <c r="B513" s="0"/>
+      <c r="C513" s="3" t="n">
+        <v>402.42</v>
+      </c>
+      <c r="D513" s="3" t="n">
+        <v>-263.17</v>
+      </c>
+    </row>
+    <row r="514" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A514" s="0"/>
+      <c r="B514" s="0"/>
+      <c r="C514" s="3" t="n">
+        <v>400.2</v>
+      </c>
+      <c r="D514" s="3" t="n">
+        <v>-266.86</v>
+      </c>
+    </row>
+    <row r="515" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A515" s="0"/>
+      <c r="B515" s="0"/>
+      <c r="C515" s="3" t="n">
+        <v>398.65</v>
+      </c>
+      <c r="D515" s="3" t="n">
+        <v>-269.9</v>
+      </c>
+    </row>
+    <row r="516" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A516" s="0"/>
+      <c r="B516" s="0"/>
+      <c r="C516" s="3" t="n">
+        <v>396.35</v>
+      </c>
+      <c r="D516" s="3" t="n">
+        <v>-273</v>
+      </c>
+    </row>
+    <row r="517" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A517" s="0"/>
+      <c r="B517" s="0"/>
+      <c r="C517" s="3" t="n">
+        <v>393.46</v>
+      </c>
+      <c r="D517" s="3" t="n">
+        <v>-276.27</v>
+      </c>
+    </row>
+    <row r="518" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A518" s="0"/>
+      <c r="B518" s="0"/>
+      <c r="C518" s="3" t="n">
+        <v>390.92</v>
+      </c>
+      <c r="D518" s="3" t="n">
+        <v>-276.94</v>
+      </c>
+    </row>
+    <row r="519" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A519" s="0"/>
+      <c r="B519" s="0"/>
+      <c r="C519" s="3" t="n">
+        <v>392.68</v>
+      </c>
+      <c r="D519" s="3" t="n">
+        <v>-273.18</v>
+      </c>
+    </row>
+    <row r="520" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A520" s="0"/>
+      <c r="B520" s="0"/>
+      <c r="C520" s="3" t="n">
+        <v>395.22</v>
+      </c>
+      <c r="D520" s="3" t="n">
+        <v>-269.43</v>
+      </c>
+    </row>
+    <row r="521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A521" s="0"/>
+      <c r="B521" s="0"/>
+      <c r="C521" s="3" t="n">
+        <v>397.98</v>
+      </c>
+      <c r="D521" s="3" t="n">
+        <v>-265.13</v>
+      </c>
+    </row>
+    <row r="522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A522" s="0"/>
+      <c r="B522" s="0"/>
+      <c r="C522" s="3" t="n">
+        <v>398.86</v>
+      </c>
+      <c r="D522" s="3" t="n">
+        <v>-261.27</v>
+      </c>
+    </row>
+    <row r="523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A523" s="0"/>
+      <c r="B523" s="0"/>
+      <c r="C523" s="3" t="n">
+        <v>398.97</v>
+      </c>
+      <c r="D523" s="3" t="n">
+        <v>-256.74</v>
+      </c>
+    </row>
+    <row r="524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A524" s="0"/>
+      <c r="B524" s="0"/>
+      <c r="C524" s="3" t="n">
+        <v>398.75</v>
+      </c>
+      <c r="D524" s="3" t="n">
+        <v>-252.66</v>
+      </c>
+    </row>
+    <row r="525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A525" s="0"/>
+      <c r="B525" s="0"/>
+      <c r="C525" s="3" t="n">
+        <v>397.43</v>
+      </c>
+      <c r="D525" s="3" t="n">
+        <v>-247.59</v>
+      </c>
+    </row>
+    <row r="526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A526" s="0"/>
+      <c r="B526" s="0"/>
+      <c r="C526" s="3" t="n">
+        <v>395.99</v>
+      </c>
+      <c r="D526" s="3" t="n">
+        <v>-243.28</v>
+      </c>
+    </row>
+    <row r="527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A527" s="0"/>
+      <c r="B527" s="0"/>
+      <c r="C527" s="3" t="n">
+        <v>394.45</v>
+      </c>
+      <c r="D527" s="3" t="n">
+        <v>-238.98</v>
+      </c>
+    </row>
+    <row r="528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A528" s="0"/>
+      <c r="B528" s="0"/>
+      <c r="C528" s="3" t="n">
+        <v>392.46</v>
+      </c>
+      <c r="D528" s="3" t="n">
+        <v>-235.89</v>
+      </c>
+    </row>
+    <row r="529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A529" s="0"/>
+      <c r="B529" s="0"/>
+      <c r="C529" s="3" t="n">
+        <v>389.37</v>
+      </c>
+      <c r="D529" s="3" t="n">
+        <v>-232.69</v>
+      </c>
+    </row>
+    <row r="530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A530" s="0"/>
+      <c r="B530" s="0"/>
+      <c r="C530" s="3" t="n">
+        <v>387.34</v>
+      </c>
+      <c r="D530" s="3" t="n">
+        <v>-228.28</v>
+      </c>
+    </row>
+    <row r="531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A531" s="0"/>
+      <c r="B531" s="0"/>
+      <c r="C531" s="3" t="n">
+        <v>384.79</v>
+      </c>
+      <c r="D531" s="3" t="n">
+        <v>-224.92</v>
+      </c>
+    </row>
+    <row r="532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A532" s="0"/>
+      <c r="B532" s="0"/>
+      <c r="C532" s="3" t="n">
+        <v>381.03</v>
+      </c>
+      <c r="D532" s="3" t="n">
+        <v>-221.97</v>
+      </c>
+    </row>
+    <row r="533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A533" s="0"/>
+      <c r="B533" s="0"/>
+      <c r="C533" s="3" t="n">
+        <v>377</v>
+      </c>
+      <c r="D533" s="3" t="n">
+        <v>-219.15</v>
+      </c>
+    </row>
+    <row r="534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A534" s="0"/>
+      <c r="B534" s="0"/>
+      <c r="C534" s="3" t="n">
+        <v>374.58</v>
+      </c>
+      <c r="D534" s="3" t="n">
+        <v>-217.27</v>
+      </c>
+    </row>
+    <row r="535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A535" s="0"/>
+      <c r="B535" s="0"/>
+      <c r="C535" s="3" t="n">
+        <v>372.16</v>
+      </c>
+      <c r="D535" s="3" t="n">
+        <v>-214.98</v>
+      </c>
+    </row>
+    <row r="536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A536" s="0"/>
+      <c r="B536" s="0"/>
+      <c r="C536" s="3" t="n">
+        <v>368.94</v>
+      </c>
+      <c r="D536" s="3" t="n">
+        <v>-211.9</v>
+      </c>
+    </row>
+    <row r="537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A537" s="0"/>
+      <c r="B537" s="0"/>
+      <c r="C537" s="3" t="n">
+        <v>364.64</v>
+      </c>
+      <c r="D537" s="3" t="n">
+        <v>-208.4</v>
+      </c>
+    </row>
+    <row r="538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A538" s="0"/>
+      <c r="B538" s="0"/>
+      <c r="C538" s="3" t="n">
+        <v>359.01</v>
+      </c>
+      <c r="D538" s="3" t="n">
+        <v>-202.36</v>
+      </c>
+    </row>
+    <row r="539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A539" s="0"/>
+      <c r="B539" s="0"/>
+      <c r="C539" s="3" t="n">
+        <v>353.23</v>
+      </c>
+      <c r="D539" s="3" t="n">
+        <v>-194.98</v>
+      </c>
+    </row>
+    <row r="540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A540" s="0"/>
+      <c r="B540" s="0"/>
+      <c r="C540" s="3" t="n">
+        <v>344.5</v>
+      </c>
+      <c r="D540" s="3" t="n">
+        <v>-181.41</v>
+      </c>
+    </row>
+    <row r="541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A541" s="0"/>
+      <c r="B541" s="0"/>
+      <c r="C541" s="3" t="n">
+        <v>340.18</v>
+      </c>
+      <c r="D541" s="3" t="n">
+        <v>-168.14</v>
+      </c>
+    </row>
+    <row r="542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A542" s="0"/>
+      <c r="B542" s="0"/>
+      <c r="C542" s="3" t="n">
+        <v>338.64</v>
+      </c>
+      <c r="D542" s="3" t="n">
+        <v>-163.14</v>
+      </c>
+    </row>
+    <row r="543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A543" s="0"/>
+      <c r="B543" s="0"/>
+      <c r="C543" s="3" t="n">
+        <v>336.66</v>
+      </c>
+      <c r="D543" s="3" t="n">
+        <v>-154.31</v>
+      </c>
+    </row>
+    <row r="544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A544" s="0"/>
+      <c r="B544" s="0"/>
+      <c r="C544" s="3" t="n">
+        <v>334.72</v>
+      </c>
+      <c r="D544" s="3" t="n">
+        <v>-161.55</v>
+      </c>
+    </row>
+    <row r="545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A545" s="0"/>
+      <c r="B545" s="0"/>
+      <c r="C545" s="3" t="n">
         <v>333.18</v>
       </c>
-      <c r="F378" s="3" t="n">
+      <c r="D545" s="3" t="n">
         <v>-166.84</v>
       </c>
     </row>
-    <row r="379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E379" s="3" t="n">
+    <row r="546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A546" s="0"/>
+      <c r="B546" s="0"/>
+      <c r="C546" s="3" t="n">
         <v>324</v>
       </c>
-      <c r="F379" s="3" t="n">
+      <c r="D546" s="3" t="n">
         <v>-187.17</v>
       </c>
     </row>
-    <row r="380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E380" s="3" t="n">
+    <row r="547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A547" s="0"/>
+      <c r="B547" s="0"/>
+      <c r="C547" s="3" t="n">
         <v>314.16</v>
       </c>
-      <c r="F380" s="3" t="n">
+      <c r="D547" s="3" t="n">
         <v>-206.4</v>
       </c>
     </row>
-    <row r="381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E381" s="3" t="n">
+    <row r="548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A548" s="0"/>
+      <c r="B548" s="0"/>
+      <c r="C548" s="3" t="n">
         <v>309.02</v>
       </c>
-      <c r="F381" s="3" t="n">
+      <c r="D548" s="3" t="n">
         <v>-215.23</v>
       </c>
     </row>
-    <row r="382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E382" s="3" t="n">
+    <row r="549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A549" s="0"/>
+      <c r="B549" s="0"/>
+      <c r="C549" s="3" t="n">
         <v>307.03</v>
       </c>
-      <c r="F382" s="3" t="n">
+      <c r="D549" s="3" t="n">
         <v>-218.95</v>
       </c>
     </row>
-    <row r="383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E383" s="3" t="n">
+    <row r="550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A550" s="0"/>
+      <c r="B550" s="0"/>
+      <c r="C550" s="3" t="n">
         <v>308.94</v>
       </c>
-      <c r="F383" s="3" t="n">
+      <c r="D550" s="3" t="n">
         <v>-231.82</v>
       </c>
     </row>
-    <row r="384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E384" s="3" t="n">
+    <row r="551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A551" s="0"/>
+      <c r="B551" s="0"/>
+      <c r="C551" s="3" t="n">
         <v>313.07</v>
       </c>
-      <c r="F384" s="3" t="n">
+      <c r="D551" s="3" t="n">
         <v>-246.43</v>
       </c>
     </row>
-    <row r="385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E385" s="3" t="n">
+    <row r="552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A552" s="0"/>
+      <c r="B552" s="0"/>
+      <c r="C552" s="3" t="n">
         <v>320</v>
       </c>
-      <c r="F385" s="3" t="n">
+      <c r="D552" s="3" t="n">
         <v>-260</v>
       </c>
     </row>
-    <row r="386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E386" s="3" t="n">
+    <row r="553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A553" s="0"/>
+      <c r="B553" s="0"/>
+      <c r="C553" s="3" t="n">
         <v>326.04</v>
       </c>
-      <c r="F386" s="3" t="n">
+      <c r="D553" s="3" t="n">
         <v>-270.89</v>
       </c>
     </row>
-    <row r="387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E387" s="3" t="n">
+    <row r="554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A554" s="0"/>
+      <c r="B554" s="0"/>
+      <c r="C554" s="3" t="n">
         <v>331.78</v>
       </c>
-      <c r="F387" s="3" t="n">
+      <c r="D554" s="3" t="n">
         <v>-277.12</v>
       </c>
     </row>
-    <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E388" s="3" t="n">
+    <row r="555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A555" s="0"/>
+      <c r="B555" s="0"/>
+      <c r="C555" s="3" t="n">
         <v>323.39</v>
       </c>
-      <c r="F388" s="3" t="n">
+      <c r="D555" s="3" t="n">
         <v>-273.61</v>
       </c>
     </row>
-    <row r="389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E389" s="3" t="n">
+    <row r="556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A556" s="0"/>
+      <c r="B556" s="0"/>
+      <c r="C556" s="3" t="n">
         <v>316.14</v>
       </c>
-      <c r="F389" s="3" t="n">
+      <c r="D556" s="3" t="n">
         <v>-267.02</v>
       </c>
     </row>
-    <row r="390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E390" s="3" t="n">
+    <row r="557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A557" s="0"/>
+      <c r="B557" s="0"/>
+      <c r="C557" s="3" t="n">
         <v>309.55</v>
       </c>
-      <c r="F390" s="3" t="n">
+      <c r="D557" s="3" t="n">
         <v>-254.93</v>
       </c>
     </row>
-    <row r="391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E391" s="3" t="n">
+    <row r="558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A558" s="0"/>
+      <c r="B558" s="0"/>
+      <c r="C558" s="3" t="n">
         <v>311.53</v>
       </c>
-      <c r="F391" s="3" t="n">
+      <c r="D558" s="3" t="n">
         <v>-271.63</v>
       </c>
     </row>
-    <row r="392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E392" s="3" t="n">
+    <row r="559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A559" s="0"/>
+      <c r="B559" s="0"/>
+      <c r="C559" s="3" t="n">
         <v>316.6</v>
       </c>
-      <c r="F392" s="3" t="n">
+      <c r="D559" s="3" t="n">
         <v>-288.03</v>
       </c>
     </row>
-    <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E393" s="3" t="n">
+    <row r="560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A560" s="0"/>
+      <c r="B560" s="0"/>
+      <c r="C560" s="3" t="n">
         <v>319.47</v>
       </c>
-      <c r="F393" s="3" t="n">
+      <c r="D560" s="3" t="n">
         <v>-295.49</v>
       </c>
     </row>
-    <row r="394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E394" s="3" t="n">
+    <row r="561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A561" s="0"/>
+      <c r="B561" s="0"/>
+      <c r="C561" s="3" t="n">
         <v>324.06</v>
       </c>
-      <c r="F394" s="3" t="n">
+      <c r="D561" s="3" t="n">
         <v>-303.72</v>
       </c>
     </row>
-    <row r="395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E395" s="3" t="n">
+    <row r="562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A562" s="0"/>
+      <c r="B562" s="0"/>
+      <c r="C562" s="3" t="n">
         <v>328.65</v>
       </c>
-      <c r="F395" s="3" t="n">
+      <c r="D562" s="3" t="n">
         <v>-311.38</v>
       </c>
     </row>
-    <row r="396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E396" s="3" t="n">
+    <row r="563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A563" s="0"/>
+      <c r="B563" s="0"/>
+      <c r="C563" s="3" t="n">
         <v>333.06</v>
       </c>
-      <c r="F396" s="3" t="n">
+      <c r="D563" s="3" t="n">
         <v>-316.55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Commit 10.1. Audio. Animacion brazo 66%. IU nueva.
</commit_message>
<xml_diff>
--- a/capas.xlsx
+++ b/capas.xlsx
@@ -43,7 +43,7 @@
     <t xml:space="preserve">TIPO</t>
   </si>
   <si>
-    <t xml:space="preserve">LINE</t>
+    <t xml:space="preserve">BACKGROUND</t>
   </si>
   <si>
     <t xml:space="preserve">COLOR</t>
@@ -70,10 +70,10 @@
     <t xml:space="preserve">OMBROS</t>
   </si>
   <si>
-    <t xml:space="preserve">BACKGROUND</t>
+    <t xml:space="preserve">#E5C1A7</t>
   </si>
   <si>
-    <t xml:space="preserve">#E5C1A7</t>
+    <t xml:space="preserve">LINE</t>
   </si>
   <si>
     <t xml:space="preserve">#00000</t>
@@ -828,13 +828,13 @@
         <v>2</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E2" s="8" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -842,13 +842,13 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>4</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1114,7 +1114,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1128,7 +1128,7 @@
         <v>4</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1178,7 +1178,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E27" s="8" t="n">
         <v>177.3</v>
@@ -1310,7 +1310,7 @@
         <v>2</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1324,7 +1324,7 @@
         <v>4</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1816,7 +1816,7 @@
         <v>2</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3083,7 +3083,7 @@
         <v>2</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3473,7 +3473,7 @@
         <v>2</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3726,7 +3726,7 @@
         <v>2</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3969,7 +3969,7 @@
         <v>2</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4090,7 +4090,7 @@
         <v>2</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4278,7 +4278,7 @@
         <v>2</v>
       </c>
       <c r="J110" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5325,7 +5325,7 @@
         <v>2</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6557,7 +6557,7 @@
         <v>2</v>
       </c>
       <c r="E385" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7973,7 +7973,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8081,7 +8081,7 @@
         <v>2</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D15" s="5"/>
     </row>
@@ -8179,7 +8179,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="4"/>
@@ -8295,7 +8295,7 @@
         <v>2</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8446,7 +8446,7 @@
         <v>2</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8543,7 +8543,7 @@
         <v>2</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8638,7 +8638,7 @@
         <v>2</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C79" s="5"/>
     </row>
@@ -8717,7 +8717,7 @@
         <v>2</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C88" s="5"/>
     </row>
@@ -8857,7 +8857,7 @@
         <v>2</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8955,7 +8955,7 @@
         <v>2</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
@@ -9055,7 +9055,7 @@
         <v>2</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C128" s="5"/>
     </row>
@@ -9141,7 +9141,7 @@
         <v>2</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9276,7 +9276,7 @@
         <v>2</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9361,7 +9361,7 @@
         <v>2</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C163" s="5"/>
     </row>
@@ -9441,7 +9441,7 @@
         <v>2</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9505,7 +9505,7 @@
         <v>2</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9593,7 +9593,7 @@
         <v>2</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9675,7 +9675,7 @@
         <v>2</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9757,7 +9757,7 @@
         <v>2</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9813,7 +9813,7 @@
         <v>2</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9923,7 +9923,7 @@
         <v>2</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C231" s="5"/>
     </row>
@@ -10040,7 +10040,7 @@
         <v>2</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10135,7 +10135,7 @@
         <v>2</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C255" s="5"/>
     </row>
@@ -10215,7 +10215,7 @@
         <v>2</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10303,7 +10303,7 @@
         <v>2</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10386,7 +10386,7 @@
         <v>2</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C284" s="5"/>
     </row>
@@ -10471,7 +10471,7 @@
         <v>2</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10528,7 +10528,7 @@
         <v>2</v>
       </c>
       <c r="B301" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10920,7 +10920,7 @@
         <v>2</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11136,7 +11136,7 @@
         <v>2</v>
       </c>
       <c r="B377" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11216,7 +11216,7 @@
         <v>2</v>
       </c>
       <c r="B387" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11778,7 +11778,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
@@ -11788,7 +11788,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -12014,7 +12014,7 @@
         <v>2</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
@@ -12266,7 +12266,7 @@
         <v>2</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -12278,7 +12278,7 @@
         <v>4</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
@@ -12381,7 +12381,7 @@
         <v>2</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="G52" s="8"/>
     </row>
@@ -12502,7 +12502,7 @@
         <v>2</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C61" s="8"/>
       <c r="D61" s="8"/>
@@ -12648,7 +12648,7 @@
         <v>2</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C73" s="8"/>
       <c r="D73" s="8"/>
@@ -12804,7 +12804,7 @@
         <v>2</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C86" s="8"/>
       <c r="D86" s="8"/>
@@ -12816,7 +12816,7 @@
         <v>4</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C87" s="8"/>
       <c r="D87" s="8"/>
@@ -13012,7 +13012,7 @@
         <v>2</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13153,7 +13153,7 @@
         <v>2</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D122" s="8"/>
       <c r="E122" s="8"/>
@@ -13345,7 +13345,7 @@
         <v>2</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D141" s="8"/>
       <c r="E141" s="8"/>
@@ -13485,7 +13485,7 @@
         <v>2</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13938,7 +13938,7 @@
         <v>2</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14203,7 +14203,7 @@
         <v>2</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14460,7 +14460,7 @@
         <v>2</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14685,7 +14685,7 @@
         <v>2</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14869,7 +14869,7 @@
         <v>2</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15086,7 +15086,7 @@
         <v>2</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15262,7 +15262,7 @@
         <v>2</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15447,7 +15447,7 @@
         <v>2</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15519,7 +15519,7 @@
         <v>2</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15696,7 +15696,7 @@
         <v>2</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15760,7 +15760,7 @@
         <v>2</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15832,7 +15832,7 @@
         <v>2</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15942,7 +15942,7 @@
         <v>2</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D268" s="1"/>
       <c r="E268" s="1"/>
@@ -16046,7 +16046,7 @@
         <v>2</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16863,7 +16863,7 @@
         <v>2</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -19273,7 +19273,7 @@
         <v>2</v>
       </c>
       <c r="B346" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19521,7 +19521,7 @@
         <v>2</v>
       </c>
       <c r="B377" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19641,7 +19641,7 @@
         <v>2</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19697,7 +19697,7 @@
         <v>2</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19761,7 +19761,7 @@
         <v>2</v>
       </c>
       <c r="B407" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19881,7 +19881,7 @@
         <v>2</v>
       </c>
       <c r="B422" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20009,7 +20009,7 @@
         <v>2</v>
       </c>
       <c r="B438" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20081,7 +20081,7 @@
         <v>2</v>
       </c>
       <c r="B447" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20153,7 +20153,7 @@
         <v>2</v>
       </c>
       <c r="B456" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20225,7 +20225,7 @@
         <v>2</v>
       </c>
       <c r="B465" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20521,7 +20521,7 @@
         <v>2</v>
       </c>
       <c r="B502" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20585,7 +20585,7 @@
         <v>2</v>
       </c>
       <c r="B510" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="511" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20649,7 +20649,7 @@
         <v>2</v>
       </c>
       <c r="B518" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="519" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22201,7 +22201,7 @@
         <v>2</v>
       </c>
       <c r="B714" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="715" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22281,7 +22281,7 @@
         <v>2</v>
       </c>
       <c r="B724" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="725" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22361,7 +22361,7 @@
         <v>2</v>
       </c>
       <c r="B734" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="735" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22537,7 +22537,7 @@
         <v>2</v>
       </c>
       <c r="B756" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="757" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22609,7 +22609,7 @@
         <v>2</v>
       </c>
       <c r="B765" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="766" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22793,7 +22793,7 @@
         <v>2</v>
       </c>
       <c r="B788" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="789" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22887,7 +22887,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22951,7 +22951,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23159,7 +23159,7 @@
         <v>2</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23253,7 +23253,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23389,7 +23389,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23541,7 +23541,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23549,7 +23549,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23781,7 +23781,7 @@
         <v>2</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23901,7 +23901,7 @@
         <v>2</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24055,7 +24055,7 @@
         <v>2</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24063,7 +24063,7 @@
         <v>4</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24415,7 +24415,7 @@
         <v>2</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24599,7 +24599,7 @@
         <v>2</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24813,7 +24813,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25045,7 +25045,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25625,7 +25625,7 @@
         <v>2</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>